<commit_message>
Update dataset (2020 SSM checked data)
</commit_message>
<xml_diff>
--- a/Dataset/2020_SSM_[checked].xlsx
+++ b/Dataset/2020_SSM_[checked].xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\filow\Desktop\Repository\LLM-EVAL-Education\Dataset\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E625D80B-222C-4936-A0D4-1D20D5961982}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA746066-03C3-41C3-A7C0-2B8C413B8E38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="16230" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -760,9 +760,6 @@
     <t>Ritmo sinusale con emiblocco fascicolare</t>
   </si>
   <si>
-    <t>Si</t>
-  </si>
-  <si>
     <t>ECG tracing</t>
   </si>
   <si>
@@ -3170,6 +3167,9 @@
   </si>
   <si>
     <t>Image Category</t>
+  </si>
+  <si>
+    <t>Yes</t>
   </si>
 </sst>
 </file>
@@ -3560,37 +3560,37 @@
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="1" t="s">
+        <v>966</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>967</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>968</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>969</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>970</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>971</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>972</v>
       </c>
-      <c r="G1" s="1" t="s">
-        <v>973</v>
-      </c>
       <c r="H1" s="1" t="s">
+        <v>1045</v>
+      </c>
+      <c r="I1" s="1" t="s">
         <v>1046</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>1047</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>1048</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>1049</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.55000000000000004">
@@ -3616,7 +3616,7 @@
         <v>6</v>
       </c>
       <c r="H2" t="s">
-        <v>974</v>
+        <v>973</v>
       </c>
       <c r="I2" t="s">
         <v>7</v>
@@ -3648,7 +3648,7 @@
         <v>15</v>
       </c>
       <c r="H3" t="s">
-        <v>974</v>
+        <v>973</v>
       </c>
       <c r="I3" t="s">
         <v>16</v>
@@ -3680,7 +3680,7 @@
         <v>23</v>
       </c>
       <c r="H4" t="s">
-        <v>975</v>
+        <v>974</v>
       </c>
       <c r="I4" t="s">
         <v>16</v>
@@ -3712,7 +3712,7 @@
         <v>30</v>
       </c>
       <c r="H5" t="s">
-        <v>976</v>
+        <v>975</v>
       </c>
       <c r="I5" t="s">
         <v>16</v>
@@ -3744,7 +3744,7 @@
         <v>37</v>
       </c>
       <c r="H6" t="s">
-        <v>976</v>
+        <v>975</v>
       </c>
       <c r="I6" t="s">
         <v>16</v>
@@ -3776,7 +3776,7 @@
         <v>44</v>
       </c>
       <c r="H7" t="s">
-        <v>977</v>
+        <v>976</v>
       </c>
       <c r="I7" t="s">
         <v>7</v>
@@ -3808,7 +3808,7 @@
         <v>36</v>
       </c>
       <c r="H8" t="s">
-        <v>974</v>
+        <v>973</v>
       </c>
       <c r="I8" t="s">
         <v>16</v>
@@ -3840,7 +3840,7 @@
         <v>57</v>
       </c>
       <c r="H9" t="s">
-        <v>978</v>
+        <v>977</v>
       </c>
       <c r="I9" t="s">
         <v>16</v>
@@ -3872,7 +3872,7 @@
         <v>64</v>
       </c>
       <c r="H10" t="s">
-        <v>979</v>
+        <v>978</v>
       </c>
       <c r="I10" t="s">
         <v>16</v>
@@ -3904,7 +3904,7 @@
         <v>71</v>
       </c>
       <c r="H11" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
       <c r="I11" t="s">
         <v>7</v>
@@ -3936,7 +3936,7 @@
         <v>78</v>
       </c>
       <c r="H12" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
       <c r="I12" t="s">
         <v>16</v>
@@ -3968,7 +3968,7 @@
         <v>85</v>
       </c>
       <c r="H13" t="s">
-        <v>981</v>
+        <v>980</v>
       </c>
       <c r="I13" t="s">
         <v>16</v>
@@ -4000,7 +4000,7 @@
         <v>92</v>
       </c>
       <c r="H14" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
       <c r="I14" t="s">
         <v>16</v>
@@ -4032,7 +4032,7 @@
         <v>99</v>
       </c>
       <c r="H15" t="s">
-        <v>982</v>
+        <v>981</v>
       </c>
       <c r="I15" t="s">
         <v>16</v>
@@ -4064,7 +4064,7 @@
         <v>105</v>
       </c>
       <c r="H16" t="s">
-        <v>983</v>
+        <v>982</v>
       </c>
       <c r="I16" t="s">
         <v>16</v>
@@ -4096,7 +4096,7 @@
         <v>112</v>
       </c>
       <c r="H17" t="s">
-        <v>984</v>
+        <v>983</v>
       </c>
       <c r="I17" t="s">
         <v>16</v>
@@ -4128,7 +4128,7 @@
         <v>119</v>
       </c>
       <c r="H18" t="s">
-        <v>985</v>
+        <v>984</v>
       </c>
       <c r="I18" t="s">
         <v>16</v>
@@ -4160,7 +4160,7 @@
         <v>126</v>
       </c>
       <c r="H19" t="s">
-        <v>986</v>
+        <v>985</v>
       </c>
       <c r="I19" t="s">
         <v>16</v>
@@ -4192,7 +4192,7 @@
         <v>133</v>
       </c>
       <c r="H20" t="s">
-        <v>987</v>
+        <v>986</v>
       </c>
       <c r="I20" t="s">
         <v>16</v>
@@ -4224,7 +4224,7 @@
         <v>140</v>
       </c>
       <c r="H21" t="s">
-        <v>988</v>
+        <v>987</v>
       </c>
       <c r="I21" t="s">
         <v>16</v>
@@ -4256,7 +4256,7 @@
         <v>147</v>
       </c>
       <c r="H22" t="s">
-        <v>989</v>
+        <v>988</v>
       </c>
       <c r="I22" t="s">
         <v>16</v>
@@ -4288,7 +4288,7 @@
         <v>154</v>
       </c>
       <c r="H23" t="s">
-        <v>990</v>
+        <v>989</v>
       </c>
       <c r="I23" t="s">
         <v>16</v>
@@ -4320,7 +4320,7 @@
         <v>161</v>
       </c>
       <c r="H24" t="s">
-        <v>978</v>
+        <v>977</v>
       </c>
       <c r="I24" t="s">
         <v>16</v>
@@ -4352,7 +4352,7 @@
         <v>168</v>
       </c>
       <c r="H25" t="s">
-        <v>978</v>
+        <v>977</v>
       </c>
       <c r="I25" t="s">
         <v>16</v>
@@ -4384,7 +4384,7 @@
         <v>175</v>
       </c>
       <c r="H26" t="s">
-        <v>978</v>
+        <v>977</v>
       </c>
       <c r="I26" t="s">
         <v>16</v>
@@ -4416,7 +4416,7 @@
         <v>182</v>
       </c>
       <c r="H27" t="s">
-        <v>991</v>
+        <v>990</v>
       </c>
       <c r="I27" t="s">
         <v>16</v>
@@ -4448,7 +4448,7 @@
         <v>189</v>
       </c>
       <c r="H28" t="s">
-        <v>991</v>
+        <v>990</v>
       </c>
       <c r="I28" t="s">
         <v>7</v>
@@ -4480,7 +4480,7 @@
         <v>196</v>
       </c>
       <c r="H29" t="s">
-        <v>992</v>
+        <v>991</v>
       </c>
       <c r="I29" t="s">
         <v>7</v>
@@ -4512,7 +4512,7 @@
         <v>203</v>
       </c>
       <c r="H30" t="s">
-        <v>993</v>
+        <v>992</v>
       </c>
       <c r="I30" t="s">
         <v>16</v>
@@ -4544,7 +4544,7 @@
         <v>210</v>
       </c>
       <c r="H31" t="s">
-        <v>994</v>
+        <v>993</v>
       </c>
       <c r="I31" t="s">
         <v>16</v>
@@ -4576,7 +4576,7 @@
         <v>217</v>
       </c>
       <c r="H32" t="s">
-        <v>994</v>
+        <v>993</v>
       </c>
       <c r="I32" t="s">
         <v>16</v>
@@ -4608,7 +4608,7 @@
         <v>224</v>
       </c>
       <c r="H33" t="s">
-        <v>994</v>
+        <v>993</v>
       </c>
       <c r="I33" t="s">
         <v>16</v>
@@ -4640,7 +4640,7 @@
         <v>231</v>
       </c>
       <c r="H34" t="s">
-        <v>976</v>
+        <v>975</v>
       </c>
       <c r="I34" t="s">
         <v>16</v>
@@ -4672,7 +4672,7 @@
         <v>238</v>
       </c>
       <c r="H35" t="s">
-        <v>976</v>
+        <v>975</v>
       </c>
       <c r="I35" t="s">
         <v>16</v>
@@ -4704,77 +4704,77 @@
         <v>245</v>
       </c>
       <c r="H36" t="s">
-        <v>976</v>
+        <v>975</v>
       </c>
       <c r="I36" t="s">
         <v>16</v>
       </c>
       <c r="J36" t="s">
+        <v>1049</v>
+      </c>
+      <c r="K36" t="s">
         <v>246</v>
-      </c>
-      <c r="K36" t="s">
-        <v>247</v>
       </c>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A37" t="s">
+        <v>247</v>
+      </c>
+      <c r="B37" t="s">
         <v>248</v>
       </c>
-      <c r="B37" t="s">
+      <c r="C37" t="s">
         <v>249</v>
       </c>
-      <c r="C37" t="s">
+      <c r="D37" t="s">
         <v>250</v>
       </c>
-      <c r="D37" t="s">
+      <c r="E37" t="s">
         <v>251</v>
       </c>
-      <c r="E37" t="s">
+      <c r="F37" t="s">
         <v>252</v>
       </c>
-      <c r="F37" t="s">
+      <c r="G37" t="s">
         <v>253</v>
       </c>
-      <c r="G37" t="s">
-        <v>254</v>
-      </c>
       <c r="H37" t="s">
-        <v>975</v>
+        <v>974</v>
       </c>
       <c r="I37" t="s">
         <v>16</v>
       </c>
       <c r="J37" t="s">
+        <v>1049</v>
+      </c>
+      <c r="K37" t="s">
         <v>246</v>
-      </c>
-      <c r="K37" t="s">
-        <v>247</v>
       </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A38" t="s">
+        <v>254</v>
+      </c>
+      <c r="B38" t="s">
         <v>255</v>
       </c>
-      <c r="B38" t="s">
+      <c r="C38" t="s">
         <v>256</v>
       </c>
-      <c r="C38" t="s">
+      <c r="D38" t="s">
         <v>257</v>
       </c>
-      <c r="D38" t="s">
+      <c r="E38" t="s">
         <v>258</v>
       </c>
-      <c r="E38" t="s">
+      <c r="F38" t="s">
         <v>259</v>
       </c>
-      <c r="F38" t="s">
+      <c r="G38" t="s">
         <v>260</v>
       </c>
-      <c r="G38" t="s">
-        <v>261</v>
-      </c>
       <c r="H38" t="s">
-        <v>976</v>
+        <v>975</v>
       </c>
       <c r="I38" t="s">
         <v>16</v>
@@ -4785,28 +4785,28 @@
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A39" t="s">
+        <v>261</v>
+      </c>
+      <c r="B39" t="s">
         <v>262</v>
       </c>
-      <c r="B39" t="s">
+      <c r="C39" t="s">
         <v>263</v>
       </c>
-      <c r="C39" t="s">
+      <c r="D39" t="s">
         <v>264</v>
       </c>
-      <c r="D39" t="s">
+      <c r="E39" t="s">
         <v>265</v>
       </c>
-      <c r="E39" t="s">
+      <c r="F39" t="s">
         <v>266</v>
       </c>
-      <c r="F39" t="s">
+      <c r="G39" t="s">
         <v>267</v>
       </c>
-      <c r="G39" t="s">
-        <v>268</v>
-      </c>
       <c r="H39" t="s">
-        <v>976</v>
+        <v>975</v>
       </c>
       <c r="I39" t="s">
         <v>16</v>
@@ -4817,28 +4817,28 @@
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A40" t="s">
+        <v>268</v>
+      </c>
+      <c r="B40" t="s">
         <v>269</v>
       </c>
-      <c r="B40" t="s">
+      <c r="C40" t="s">
         <v>270</v>
       </c>
-      <c r="C40" t="s">
+      <c r="D40" t="s">
         <v>271</v>
       </c>
-      <c r="D40" t="s">
+      <c r="E40" t="s">
         <v>272</v>
       </c>
-      <c r="E40" t="s">
+      <c r="F40" t="s">
         <v>273</v>
       </c>
-      <c r="F40" t="s">
+      <c r="G40" t="s">
         <v>274</v>
       </c>
-      <c r="G40" t="s">
-        <v>275</v>
-      </c>
       <c r="H40" t="s">
-        <v>976</v>
+        <v>975</v>
       </c>
       <c r="I40" t="s">
         <v>16</v>
@@ -4849,28 +4849,28 @@
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A41" t="s">
+        <v>275</v>
+      </c>
+      <c r="B41" t="s">
         <v>276</v>
       </c>
-      <c r="B41" t="s">
+      <c r="C41" t="s">
         <v>277</v>
       </c>
-      <c r="C41" t="s">
+      <c r="D41" t="s">
         <v>278</v>
       </c>
-      <c r="D41" t="s">
+      <c r="E41" t="s">
         <v>279</v>
       </c>
-      <c r="E41" t="s">
+      <c r="F41" t="s">
         <v>280</v>
       </c>
-      <c r="F41" t="s">
+      <c r="G41" t="s">
         <v>281</v>
       </c>
-      <c r="G41" t="s">
-        <v>282</v>
-      </c>
       <c r="H41" t="s">
-        <v>975</v>
+        <v>974</v>
       </c>
       <c r="I41" t="s">
         <v>16</v>
@@ -4881,28 +4881,28 @@
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A42" t="s">
+        <v>282</v>
+      </c>
+      <c r="B42" t="s">
         <v>283</v>
       </c>
-      <c r="B42" t="s">
+      <c r="C42" t="s">
         <v>284</v>
       </c>
-      <c r="C42" t="s">
+      <c r="D42" t="s">
         <v>285</v>
       </c>
-      <c r="D42" t="s">
+      <c r="E42" t="s">
         <v>286</v>
       </c>
-      <c r="E42" t="s">
+      <c r="F42" t="s">
         <v>287</v>
       </c>
-      <c r="F42" t="s">
+      <c r="G42" t="s">
         <v>288</v>
       </c>
-      <c r="G42" t="s">
-        <v>289</v>
-      </c>
       <c r="H42" t="s">
-        <v>995</v>
+        <v>994</v>
       </c>
       <c r="I42" t="s">
         <v>16</v>
@@ -4913,28 +4913,28 @@
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A43" t="s">
+        <v>289</v>
+      </c>
+      <c r="B43" t="s">
         <v>290</v>
       </c>
-      <c r="B43" t="s">
+      <c r="C43" t="s">
         <v>291</v>
       </c>
-      <c r="C43" t="s">
+      <c r="D43" t="s">
         <v>292</v>
       </c>
-      <c r="D43" t="s">
+      <c r="E43" t="s">
         <v>293</v>
       </c>
-      <c r="E43" t="s">
+      <c r="F43" t="s">
         <v>294</v>
       </c>
-      <c r="F43" t="s">
+      <c r="G43" t="s">
         <v>295</v>
       </c>
-      <c r="G43" t="s">
-        <v>296</v>
-      </c>
       <c r="H43" t="s">
-        <v>975</v>
+        <v>974</v>
       </c>
       <c r="I43" t="s">
         <v>16</v>
@@ -4945,28 +4945,28 @@
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A44" t="s">
+        <v>296</v>
+      </c>
+      <c r="B44" t="s">
         <v>297</v>
       </c>
-      <c r="B44" t="s">
+      <c r="C44" t="s">
         <v>298</v>
       </c>
-      <c r="C44" t="s">
+      <c r="D44" t="s">
         <v>299</v>
       </c>
-      <c r="D44" t="s">
+      <c r="E44" t="s">
         <v>300</v>
       </c>
-      <c r="E44" t="s">
+      <c r="F44" t="s">
         <v>301</v>
       </c>
-      <c r="F44" t="s">
+      <c r="G44" t="s">
         <v>302</v>
       </c>
-      <c r="G44" t="s">
-        <v>303</v>
-      </c>
       <c r="H44" t="s">
-        <v>996</v>
+        <v>995</v>
       </c>
       <c r="I44" t="s">
         <v>16</v>
@@ -4977,28 +4977,28 @@
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A45" t="s">
+        <v>303</v>
+      </c>
+      <c r="B45" t="s">
         <v>304</v>
       </c>
-      <c r="B45" t="s">
+      <c r="C45" t="s">
         <v>305</v>
       </c>
-      <c r="C45" t="s">
+      <c r="D45" t="s">
         <v>306</v>
       </c>
-      <c r="D45" t="s">
+      <c r="E45" t="s">
         <v>307</v>
       </c>
-      <c r="E45" t="s">
+      <c r="F45" t="s">
         <v>308</v>
       </c>
-      <c r="F45" t="s">
+      <c r="G45" t="s">
         <v>309</v>
       </c>
-      <c r="G45" t="s">
-        <v>310</v>
-      </c>
       <c r="H45" t="s">
-        <v>996</v>
+        <v>995</v>
       </c>
       <c r="I45" t="s">
         <v>7</v>
@@ -5009,28 +5009,28 @@
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A46" t="s">
+        <v>310</v>
+      </c>
+      <c r="B46" t="s">
         <v>311</v>
       </c>
-      <c r="B46" t="s">
+      <c r="C46" t="s">
         <v>312</v>
       </c>
-      <c r="C46" t="s">
+      <c r="D46" t="s">
         <v>313</v>
       </c>
-      <c r="D46" t="s">
+      <c r="E46" t="s">
         <v>314</v>
       </c>
-      <c r="E46" t="s">
+      <c r="F46" t="s">
         <v>315</v>
       </c>
-      <c r="F46" t="s">
+      <c r="G46" t="s">
         <v>316</v>
       </c>
-      <c r="G46" t="s">
-        <v>317</v>
-      </c>
       <c r="H46" t="s">
-        <v>997</v>
+        <v>996</v>
       </c>
       <c r="I46" t="s">
         <v>16</v>
@@ -5041,28 +5041,28 @@
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A47" t="s">
+        <v>317</v>
+      </c>
+      <c r="B47" t="s">
         <v>318</v>
       </c>
-      <c r="B47" t="s">
+      <c r="C47" t="s">
         <v>319</v>
       </c>
-      <c r="C47" t="s">
+      <c r="D47" t="s">
         <v>320</v>
       </c>
-      <c r="D47" t="s">
+      <c r="E47" t="s">
         <v>321</v>
       </c>
-      <c r="E47" t="s">
+      <c r="F47" t="s">
         <v>322</v>
       </c>
-      <c r="F47" t="s">
+      <c r="G47" t="s">
         <v>323</v>
       </c>
-      <c r="G47" t="s">
-        <v>324</v>
-      </c>
       <c r="H47" t="s">
-        <v>997</v>
+        <v>996</v>
       </c>
       <c r="I47" t="s">
         <v>7</v>
@@ -5073,28 +5073,28 @@
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A48" t="s">
+        <v>324</v>
+      </c>
+      <c r="B48" t="s">
         <v>325</v>
       </c>
-      <c r="B48" t="s">
+      <c r="C48" t="s">
         <v>326</v>
       </c>
-      <c r="C48" t="s">
+      <c r="D48" t="s">
         <v>327</v>
       </c>
-      <c r="D48" t="s">
+      <c r="E48" t="s">
         <v>328</v>
       </c>
-      <c r="E48" t="s">
+      <c r="F48" t="s">
         <v>329</v>
       </c>
-      <c r="F48" t="s">
+      <c r="G48" t="s">
         <v>330</v>
       </c>
-      <c r="G48" t="s">
-        <v>331</v>
-      </c>
       <c r="H48" t="s">
-        <v>998</v>
+        <v>997</v>
       </c>
       <c r="I48" t="s">
         <v>16</v>
@@ -5105,28 +5105,28 @@
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A49" t="s">
+        <v>331</v>
+      </c>
+      <c r="B49" t="s">
         <v>332</v>
       </c>
-      <c r="B49" t="s">
+      <c r="C49" t="s">
         <v>333</v>
       </c>
-      <c r="C49" t="s">
+      <c r="D49" t="s">
         <v>334</v>
       </c>
-      <c r="D49" t="s">
+      <c r="E49" t="s">
         <v>335</v>
-      </c>
-      <c r="E49" t="s">
-        <v>336</v>
       </c>
       <c r="F49" t="s">
         <v>222</v>
       </c>
       <c r="G49" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="H49" t="s">
-        <v>974</v>
+        <v>973</v>
       </c>
       <c r="I49" t="s">
         <v>16</v>
@@ -5137,28 +5137,28 @@
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A50" t="s">
+        <v>337</v>
+      </c>
+      <c r="B50" t="s">
         <v>338</v>
       </c>
-      <c r="B50" t="s">
+      <c r="C50" t="s">
         <v>339</v>
       </c>
-      <c r="C50" t="s">
+      <c r="D50" t="s">
         <v>340</v>
       </c>
-      <c r="D50" t="s">
+      <c r="E50" t="s">
         <v>341</v>
       </c>
-      <c r="E50" t="s">
+      <c r="F50" t="s">
         <v>342</v>
       </c>
-      <c r="F50" t="s">
+      <c r="G50" t="s">
         <v>343</v>
       </c>
-      <c r="G50" t="s">
-        <v>344</v>
-      </c>
       <c r="H50" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
       <c r="I50" t="s">
         <v>16</v>
@@ -5169,28 +5169,28 @@
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A51" t="s">
+        <v>344</v>
+      </c>
+      <c r="B51" t="s">
         <v>345</v>
       </c>
-      <c r="B51" t="s">
+      <c r="C51" t="s">
         <v>346</v>
       </c>
-      <c r="C51" t="s">
+      <c r="D51" t="s">
         <v>347</v>
       </c>
-      <c r="D51" t="s">
+      <c r="E51" t="s">
         <v>348</v>
       </c>
-      <c r="E51" t="s">
+      <c r="F51" t="s">
         <v>349</v>
       </c>
-      <c r="F51" t="s">
+      <c r="G51" t="s">
         <v>350</v>
       </c>
-      <c r="G51" t="s">
-        <v>351</v>
-      </c>
       <c r="H51" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
       <c r="I51" t="s">
         <v>16</v>
@@ -5201,28 +5201,28 @@
     </row>
     <row r="52" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A52" t="s">
+        <v>351</v>
+      </c>
+      <c r="B52" t="s">
         <v>352</v>
       </c>
-      <c r="B52" t="s">
+      <c r="C52" t="s">
         <v>353</v>
       </c>
-      <c r="C52" t="s">
+      <c r="D52" t="s">
         <v>354</v>
       </c>
-      <c r="D52" t="s">
+      <c r="E52" t="s">
         <v>355</v>
       </c>
-      <c r="E52" t="s">
+      <c r="F52" t="s">
         <v>356</v>
       </c>
-      <c r="F52" t="s">
-        <v>357</v>
-      </c>
       <c r="G52" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="H52" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
       <c r="I52" t="s">
         <v>16</v>
@@ -5233,28 +5233,28 @@
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A53" t="s">
+        <v>357</v>
+      </c>
+      <c r="B53" t="s">
         <v>358</v>
       </c>
-      <c r="B53" t="s">
+      <c r="C53" t="s">
         <v>359</v>
       </c>
-      <c r="C53" t="s">
+      <c r="D53" t="s">
         <v>360</v>
       </c>
-      <c r="D53" t="s">
+      <c r="E53" t="s">
         <v>361</v>
       </c>
-      <c r="E53" t="s">
+      <c r="F53" t="s">
         <v>362</v>
       </c>
-      <c r="F53" t="s">
+      <c r="G53" t="s">
         <v>363</v>
       </c>
-      <c r="G53" t="s">
-        <v>364</v>
-      </c>
       <c r="H53" t="s">
-        <v>999</v>
+        <v>998</v>
       </c>
       <c r="I53" t="s">
         <v>16</v>
@@ -5265,28 +5265,28 @@
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A54" t="s">
+        <v>364</v>
+      </c>
+      <c r="B54" t="s">
         <v>365</v>
       </c>
-      <c r="B54" t="s">
+      <c r="C54" t="s">
         <v>366</v>
       </c>
-      <c r="C54" t="s">
+      <c r="D54" t="s">
         <v>367</v>
       </c>
-      <c r="D54" t="s">
+      <c r="E54" t="s">
         <v>368</v>
       </c>
-      <c r="E54" t="s">
+      <c r="F54" t="s">
         <v>369</v>
       </c>
-      <c r="F54" t="s">
+      <c r="G54" t="s">
         <v>370</v>
       </c>
-      <c r="G54" t="s">
-        <v>371</v>
-      </c>
       <c r="H54" t="s">
-        <v>1000</v>
+        <v>999</v>
       </c>
       <c r="I54" t="s">
         <v>16</v>
@@ -5297,28 +5297,28 @@
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A55" t="s">
+        <v>371</v>
+      </c>
+      <c r="B55" t="s">
         <v>372</v>
       </c>
-      <c r="B55" t="s">
+      <c r="C55" t="s">
         <v>373</v>
       </c>
-      <c r="C55" t="s">
+      <c r="D55" t="s">
         <v>374</v>
       </c>
-      <c r="D55" t="s">
+      <c r="E55" t="s">
         <v>375</v>
       </c>
-      <c r="E55" t="s">
+      <c r="F55" t="s">
         <v>376</v>
       </c>
-      <c r="F55" t="s">
+      <c r="G55" t="s">
         <v>377</v>
       </c>
-      <c r="G55" t="s">
-        <v>378</v>
-      </c>
       <c r="H55" t="s">
-        <v>1000</v>
+        <v>999</v>
       </c>
       <c r="I55" t="s">
         <v>16</v>
@@ -5329,28 +5329,28 @@
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A56" t="s">
+        <v>378</v>
+      </c>
+      <c r="B56" t="s">
         <v>379</v>
       </c>
-      <c r="B56" t="s">
+      <c r="C56" t="s">
         <v>380</v>
       </c>
-      <c r="C56" t="s">
+      <c r="D56" t="s">
         <v>381</v>
       </c>
-      <c r="D56" t="s">
+      <c r="E56" t="s">
         <v>382</v>
       </c>
-      <c r="E56" t="s">
+      <c r="F56" t="s">
         <v>383</v>
       </c>
-      <c r="F56" t="s">
+      <c r="G56" t="s">
         <v>384</v>
       </c>
-      <c r="G56" t="s">
-        <v>385</v>
-      </c>
       <c r="H56" t="s">
-        <v>1001</v>
+        <v>1000</v>
       </c>
       <c r="I56" t="s">
         <v>16</v>
@@ -5361,28 +5361,28 @@
     </row>
     <row r="57" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A57" t="s">
+        <v>385</v>
+      </c>
+      <c r="B57" t="s">
         <v>386</v>
       </c>
-      <c r="B57" t="s">
+      <c r="C57" t="s">
         <v>387</v>
       </c>
-      <c r="C57" t="s">
+      <c r="D57" t="s">
         <v>388</v>
       </c>
-      <c r="D57" t="s">
+      <c r="E57" t="s">
         <v>389</v>
       </c>
-      <c r="E57" t="s">
+      <c r="F57" t="s">
         <v>390</v>
       </c>
-      <c r="F57" t="s">
+      <c r="G57" t="s">
         <v>391</v>
       </c>
-      <c r="G57" t="s">
-        <v>392</v>
-      </c>
       <c r="H57" t="s">
-        <v>1002</v>
+        <v>1001</v>
       </c>
       <c r="I57" t="s">
         <v>7</v>
@@ -5393,28 +5393,28 @@
     </row>
     <row r="58" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A58" t="s">
+        <v>392</v>
+      </c>
+      <c r="B58" t="s">
         <v>393</v>
       </c>
-      <c r="B58" t="s">
+      <c r="C58" t="s">
         <v>394</v>
       </c>
-      <c r="C58" t="s">
+      <c r="D58" t="s">
         <v>395</v>
       </c>
-      <c r="D58" t="s">
+      <c r="E58" t="s">
         <v>396</v>
       </c>
-      <c r="E58" t="s">
+      <c r="F58" t="s">
         <v>397</v>
       </c>
-      <c r="F58" t="s">
+      <c r="G58" t="s">
         <v>398</v>
       </c>
-      <c r="G58" t="s">
-        <v>399</v>
-      </c>
       <c r="H58" t="s">
-        <v>994</v>
+        <v>993</v>
       </c>
       <c r="I58" t="s">
         <v>7</v>
@@ -5425,28 +5425,28 @@
     </row>
     <row r="59" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A59" t="s">
+        <v>399</v>
+      </c>
+      <c r="B59" t="s">
         <v>400</v>
       </c>
-      <c r="B59" t="s">
+      <c r="C59" t="s">
         <v>401</v>
       </c>
-      <c r="C59" t="s">
+      <c r="D59" t="s">
         <v>402</v>
       </c>
-      <c r="D59" t="s">
+      <c r="E59" t="s">
         <v>403</v>
       </c>
-      <c r="E59" t="s">
+      <c r="F59" t="s">
         <v>404</v>
       </c>
-      <c r="F59" t="s">
+      <c r="G59" t="s">
         <v>405</v>
       </c>
-      <c r="G59" t="s">
-        <v>406</v>
-      </c>
       <c r="H59" t="s">
-        <v>1003</v>
+        <v>1002</v>
       </c>
       <c r="I59" t="s">
         <v>16</v>
@@ -5457,28 +5457,28 @@
     </row>
     <row r="60" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A60" t="s">
+        <v>406</v>
+      </c>
+      <c r="B60" t="s">
         <v>407</v>
       </c>
-      <c r="B60" t="s">
+      <c r="C60" t="s">
         <v>408</v>
       </c>
-      <c r="C60" t="s">
+      <c r="D60" t="s">
         <v>409</v>
       </c>
-      <c r="D60" t="s">
+      <c r="E60" t="s">
         <v>410</v>
       </c>
-      <c r="E60" t="s">
+      <c r="F60" t="s">
         <v>411</v>
       </c>
-      <c r="F60" t="s">
+      <c r="G60" t="s">
         <v>412</v>
       </c>
-      <c r="G60" t="s">
-        <v>413</v>
-      </c>
       <c r="H60" t="s">
-        <v>1004</v>
+        <v>1003</v>
       </c>
       <c r="I60" t="s">
         <v>16</v>
@@ -5489,28 +5489,28 @@
     </row>
     <row r="61" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A61" t="s">
+        <v>413</v>
+      </c>
+      <c r="B61" t="s">
         <v>414</v>
       </c>
-      <c r="B61" t="s">
+      <c r="C61" t="s">
         <v>415</v>
       </c>
-      <c r="C61" t="s">
+      <c r="D61" t="s">
         <v>416</v>
       </c>
-      <c r="D61" t="s">
+      <c r="E61" t="s">
         <v>417</v>
       </c>
-      <c r="E61" t="s">
+      <c r="F61" t="s">
         <v>418</v>
       </c>
-      <c r="F61" t="s">
+      <c r="G61" t="s">
         <v>419</v>
       </c>
-      <c r="G61" t="s">
-        <v>420</v>
-      </c>
       <c r="H61" t="s">
-        <v>1005</v>
+        <v>1004</v>
       </c>
       <c r="I61" t="s">
         <v>16</v>
@@ -5521,28 +5521,28 @@
     </row>
     <row r="62" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A62" t="s">
+        <v>420</v>
+      </c>
+      <c r="B62" t="s">
         <v>421</v>
       </c>
-      <c r="B62" t="s">
+      <c r="C62" t="s">
         <v>422</v>
       </c>
-      <c r="C62" t="s">
+      <c r="D62" t="s">
         <v>423</v>
       </c>
-      <c r="D62" t="s">
+      <c r="E62" t="s">
         <v>424</v>
       </c>
-      <c r="E62" t="s">
+      <c r="F62" t="s">
         <v>425</v>
       </c>
-      <c r="F62" t="s">
+      <c r="G62" t="s">
         <v>426</v>
       </c>
-      <c r="G62" t="s">
-        <v>427</v>
-      </c>
       <c r="H62" t="s">
-        <v>1006</v>
+        <v>1005</v>
       </c>
       <c r="I62" t="s">
         <v>16</v>
@@ -5553,28 +5553,28 @@
     </row>
     <row r="63" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A63" t="s">
+        <v>427</v>
+      </c>
+      <c r="B63" t="s">
         <v>428</v>
       </c>
-      <c r="B63" t="s">
+      <c r="C63" t="s">
         <v>429</v>
       </c>
-      <c r="C63" t="s">
+      <c r="D63" t="s">
         <v>430</v>
       </c>
-      <c r="D63" t="s">
+      <c r="E63" t="s">
         <v>431</v>
       </c>
-      <c r="E63" t="s">
+      <c r="F63" t="s">
         <v>432</v>
       </c>
-      <c r="F63" t="s">
+      <c r="G63" t="s">
         <v>433</v>
       </c>
-      <c r="G63" t="s">
-        <v>434</v>
-      </c>
       <c r="H63" t="s">
-        <v>1006</v>
+        <v>1005</v>
       </c>
       <c r="I63" t="s">
         <v>16</v>
@@ -5585,28 +5585,28 @@
     </row>
     <row r="64" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A64" t="s">
+        <v>434</v>
+      </c>
+      <c r="B64" t="s">
         <v>435</v>
       </c>
-      <c r="B64" t="s">
+      <c r="C64" t="s">
         <v>436</v>
       </c>
-      <c r="C64" t="s">
+      <c r="D64" t="s">
         <v>437</v>
       </c>
-      <c r="D64" t="s">
+      <c r="E64" t="s">
         <v>438</v>
       </c>
-      <c r="E64" t="s">
+      <c r="F64" t="s">
         <v>439</v>
       </c>
-      <c r="F64" t="s">
+      <c r="G64" t="s">
         <v>440</v>
       </c>
-      <c r="G64" t="s">
-        <v>441</v>
-      </c>
       <c r="H64" t="s">
-        <v>1007</v>
+        <v>1006</v>
       </c>
       <c r="I64" t="s">
         <v>7</v>
@@ -5617,28 +5617,28 @@
     </row>
     <row r="65" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A65" t="s">
+        <v>441</v>
+      </c>
+      <c r="B65" t="s">
         <v>442</v>
       </c>
-      <c r="B65" t="s">
+      <c r="C65" t="s">
         <v>443</v>
       </c>
-      <c r="C65" t="s">
+      <c r="D65" t="s">
         <v>444</v>
       </c>
-      <c r="D65" t="s">
+      <c r="E65" t="s">
         <v>445</v>
       </c>
-      <c r="E65" t="s">
+      <c r="F65" t="s">
         <v>446</v>
       </c>
-      <c r="F65" t="s">
-        <v>447</v>
-      </c>
       <c r="G65" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="H65" t="s">
-        <v>1008</v>
+        <v>1007</v>
       </c>
       <c r="I65" t="s">
         <v>7</v>
@@ -5649,28 +5649,28 @@
     </row>
     <row r="66" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A66" t="s">
+        <v>447</v>
+      </c>
+      <c r="B66" t="s">
         <v>448</v>
       </c>
-      <c r="B66" t="s">
+      <c r="C66" t="s">
         <v>449</v>
       </c>
-      <c r="C66" t="s">
+      <c r="D66" t="s">
         <v>450</v>
       </c>
-      <c r="D66" t="s">
+      <c r="E66" t="s">
         <v>451</v>
       </c>
-      <c r="E66" t="s">
+      <c r="F66" t="s">
         <v>452</v>
       </c>
-      <c r="F66" t="s">
+      <c r="G66" t="s">
         <v>453</v>
       </c>
-      <c r="G66" t="s">
-        <v>454</v>
-      </c>
       <c r="H66" t="s">
-        <v>994</v>
+        <v>993</v>
       </c>
       <c r="I66" t="s">
         <v>16</v>
@@ -5681,28 +5681,28 @@
     </row>
     <row r="67" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A67" t="s">
+        <v>454</v>
+      </c>
+      <c r="B67" t="s">
         <v>455</v>
       </c>
-      <c r="B67" t="s">
+      <c r="C67" t="s">
         <v>456</v>
       </c>
-      <c r="C67" t="s">
+      <c r="D67" t="s">
         <v>457</v>
       </c>
-      <c r="D67" t="s">
+      <c r="E67" t="s">
         <v>458</v>
       </c>
-      <c r="E67" t="s">
+      <c r="F67" t="s">
         <v>459</v>
       </c>
-      <c r="F67" t="s">
+      <c r="G67" t="s">
         <v>460</v>
       </c>
-      <c r="G67" t="s">
-        <v>461</v>
-      </c>
       <c r="H67" t="s">
-        <v>994</v>
+        <v>993</v>
       </c>
       <c r="I67" t="s">
         <v>7</v>
@@ -5713,28 +5713,28 @@
     </row>
     <row r="68" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A68" t="s">
+        <v>461</v>
+      </c>
+      <c r="B68" t="s">
         <v>462</v>
       </c>
-      <c r="B68" t="s">
+      <c r="C68" t="s">
         <v>463</v>
       </c>
-      <c r="C68" t="s">
+      <c r="D68" t="s">
         <v>464</v>
       </c>
-      <c r="D68" t="s">
+      <c r="E68" t="s">
         <v>465</v>
       </c>
-      <c r="E68" t="s">
+      <c r="F68" t="s">
         <v>466</v>
       </c>
-      <c r="F68" t="s">
+      <c r="G68" t="s">
         <v>467</v>
       </c>
-      <c r="G68" t="s">
-        <v>468</v>
-      </c>
       <c r="H68" t="s">
-        <v>1009</v>
+        <v>1008</v>
       </c>
       <c r="I68" t="s">
         <v>7</v>
@@ -5745,28 +5745,28 @@
     </row>
     <row r="69" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A69" t="s">
+        <v>468</v>
+      </c>
+      <c r="B69" t="s">
         <v>469</v>
       </c>
-      <c r="B69" t="s">
+      <c r="C69" t="s">
         <v>470</v>
       </c>
-      <c r="C69" t="s">
+      <c r="D69" t="s">
         <v>471</v>
       </c>
-      <c r="D69" t="s">
+      <c r="E69" t="s">
         <v>472</v>
       </c>
-      <c r="E69" t="s">
+      <c r="F69" t="s">
         <v>473</v>
       </c>
-      <c r="F69" t="s">
+      <c r="G69" t="s">
         <v>474</v>
       </c>
-      <c r="G69" t="s">
-        <v>475</v>
-      </c>
       <c r="H69" t="s">
-        <v>1010</v>
+        <v>1009</v>
       </c>
       <c r="I69" t="s">
         <v>7</v>
@@ -5777,28 +5777,28 @@
     </row>
     <row r="70" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A70" t="s">
+        <v>475</v>
+      </c>
+      <c r="B70" t="s">
         <v>476</v>
       </c>
-      <c r="B70" t="s">
+      <c r="C70" t="s">
         <v>477</v>
       </c>
-      <c r="C70" t="s">
+      <c r="D70" t="s">
+        <v>451</v>
+      </c>
+      <c r="E70" t="s">
         <v>478</v>
       </c>
-      <c r="D70" t="s">
-        <v>452</v>
-      </c>
-      <c r="E70" t="s">
+      <c r="F70" t="s">
         <v>479</v>
       </c>
-      <c r="F70" t="s">
+      <c r="G70" t="s">
         <v>480</v>
       </c>
-      <c r="G70" t="s">
-        <v>481</v>
-      </c>
       <c r="H70" t="s">
-        <v>1011</v>
+        <v>1010</v>
       </c>
       <c r="I70" t="s">
         <v>16</v>
@@ -5809,28 +5809,28 @@
     </row>
     <row r="71" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A71" t="s">
+        <v>481</v>
+      </c>
+      <c r="B71" t="s">
         <v>482</v>
       </c>
-      <c r="B71" t="s">
+      <c r="C71" t="s">
         <v>483</v>
       </c>
-      <c r="C71" t="s">
+      <c r="D71" t="s">
         <v>484</v>
       </c>
-      <c r="D71" t="s">
+      <c r="E71" t="s">
         <v>485</v>
       </c>
-      <c r="E71" t="s">
+      <c r="F71" t="s">
         <v>486</v>
       </c>
-      <c r="F71" t="s">
+      <c r="G71" t="s">
         <v>487</v>
       </c>
-      <c r="G71" t="s">
-        <v>488</v>
-      </c>
       <c r="H71" t="s">
-        <v>1012</v>
+        <v>1011</v>
       </c>
       <c r="I71" t="s">
         <v>16</v>
@@ -5841,28 +5841,28 @@
     </row>
     <row r="72" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A72" t="s">
+        <v>488</v>
+      </c>
+      <c r="B72" t="s">
         <v>489</v>
       </c>
-      <c r="B72" t="s">
+      <c r="C72" t="s">
         <v>490</v>
       </c>
-      <c r="C72" t="s">
+      <c r="D72" t="s">
         <v>491</v>
       </c>
-      <c r="D72" t="s">
+      <c r="E72" t="s">
         <v>492</v>
       </c>
-      <c r="E72" t="s">
+      <c r="F72" t="s">
         <v>493</v>
       </c>
-      <c r="F72" t="s">
+      <c r="G72" t="s">
         <v>494</v>
       </c>
-      <c r="G72" t="s">
-        <v>495</v>
-      </c>
       <c r="H72" t="s">
-        <v>991</v>
+        <v>990</v>
       </c>
       <c r="I72" t="s">
         <v>16</v>
@@ -5873,28 +5873,28 @@
     </row>
     <row r="73" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A73" t="s">
+        <v>495</v>
+      </c>
+      <c r="B73" t="s">
         <v>496</v>
       </c>
-      <c r="B73" t="s">
+      <c r="C73" t="s">
         <v>497</v>
       </c>
-      <c r="C73" t="s">
+      <c r="D73" t="s">
         <v>498</v>
       </c>
-      <c r="D73" t="s">
+      <c r="E73" t="s">
         <v>499</v>
       </c>
-      <c r="E73" t="s">
+      <c r="F73" t="s">
         <v>500</v>
       </c>
-      <c r="F73" t="s">
+      <c r="G73" t="s">
         <v>501</v>
       </c>
-      <c r="G73" t="s">
-        <v>502</v>
-      </c>
       <c r="H73" t="s">
-        <v>1012</v>
+        <v>1011</v>
       </c>
       <c r="I73" t="s">
         <v>16</v>
@@ -5905,28 +5905,28 @@
     </row>
     <row r="74" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A74" t="s">
+        <v>502</v>
+      </c>
+      <c r="B74" t="s">
         <v>503</v>
       </c>
-      <c r="B74" t="s">
+      <c r="C74" t="s">
         <v>504</v>
       </c>
-      <c r="C74" t="s">
+      <c r="D74" t="s">
         <v>505</v>
       </c>
-      <c r="D74" t="s">
+      <c r="E74" t="s">
         <v>506</v>
       </c>
-      <c r="E74" t="s">
+      <c r="F74" t="s">
         <v>507</v>
       </c>
-      <c r="F74" t="s">
+      <c r="G74" t="s">
         <v>508</v>
       </c>
-      <c r="G74" t="s">
-        <v>509</v>
-      </c>
       <c r="H74" t="s">
-        <v>1013</v>
+        <v>1012</v>
       </c>
       <c r="I74" t="s">
         <v>7</v>
@@ -5937,28 +5937,28 @@
     </row>
     <row r="75" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A75" t="s">
+        <v>509</v>
+      </c>
+      <c r="B75" t="s">
         <v>510</v>
       </c>
-      <c r="B75" t="s">
+      <c r="C75" t="s">
         <v>511</v>
       </c>
-      <c r="C75" t="s">
+      <c r="D75" t="s">
         <v>512</v>
       </c>
-      <c r="D75" t="s">
+      <c r="E75" t="s">
         <v>513</v>
       </c>
-      <c r="E75" t="s">
+      <c r="F75" t="s">
         <v>514</v>
       </c>
-      <c r="F75" t="s">
+      <c r="G75" t="s">
         <v>515</v>
       </c>
-      <c r="G75" t="s">
-        <v>516</v>
-      </c>
       <c r="H75" t="s">
-        <v>1012</v>
+        <v>1011</v>
       </c>
       <c r="I75" t="s">
         <v>7</v>
@@ -5969,28 +5969,28 @@
     </row>
     <row r="76" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A76" t="s">
+        <v>516</v>
+      </c>
+      <c r="B76" t="s">
         <v>517</v>
       </c>
-      <c r="B76" t="s">
+      <c r="C76" t="s">
         <v>518</v>
       </c>
-      <c r="C76" t="s">
+      <c r="D76" t="s">
         <v>519</v>
       </c>
-      <c r="D76" t="s">
+      <c r="E76" t="s">
         <v>520</v>
       </c>
-      <c r="E76" t="s">
+      <c r="F76" t="s">
         <v>521</v>
       </c>
-      <c r="F76" t="s">
+      <c r="G76" t="s">
         <v>522</v>
       </c>
-      <c r="G76" t="s">
-        <v>523</v>
-      </c>
       <c r="H76" t="s">
-        <v>1010</v>
+        <v>1009</v>
       </c>
       <c r="I76" t="s">
         <v>7</v>
@@ -6001,28 +6001,28 @@
     </row>
     <row r="77" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A77" t="s">
+        <v>523</v>
+      </c>
+      <c r="B77" t="s">
         <v>524</v>
       </c>
-      <c r="B77" t="s">
+      <c r="C77" t="s">
         <v>525</v>
       </c>
-      <c r="C77" t="s">
+      <c r="D77" t="s">
         <v>526</v>
       </c>
-      <c r="D77" t="s">
+      <c r="E77" t="s">
         <v>527</v>
       </c>
-      <c r="E77" t="s">
+      <c r="F77" t="s">
         <v>528</v>
       </c>
-      <c r="F77" t="s">
-        <v>529</v>
-      </c>
       <c r="G77" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="H77" t="s">
-        <v>1014</v>
+        <v>1013</v>
       </c>
       <c r="I77" t="s">
         <v>7</v>
@@ -6033,28 +6033,28 @@
     </row>
     <row r="78" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A78" t="s">
+        <v>529</v>
+      </c>
+      <c r="B78" t="s">
         <v>530</v>
       </c>
-      <c r="B78" t="s">
+      <c r="C78" t="s">
         <v>531</v>
       </c>
-      <c r="C78" t="s">
+      <c r="D78" t="s">
         <v>532</v>
       </c>
-      <c r="D78" t="s">
+      <c r="E78" t="s">
         <v>533</v>
       </c>
-      <c r="E78" t="s">
+      <c r="F78" t="s">
         <v>534</v>
       </c>
-      <c r="F78" t="s">
+      <c r="G78" t="s">
         <v>535</v>
       </c>
-      <c r="G78" t="s">
-        <v>536</v>
-      </c>
       <c r="H78" t="s">
-        <v>1010</v>
+        <v>1009</v>
       </c>
       <c r="I78" t="s">
         <v>7</v>
@@ -6065,28 +6065,28 @@
     </row>
     <row r="79" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A79" t="s">
+        <v>536</v>
+      </c>
+      <c r="B79" t="s">
         <v>537</v>
       </c>
-      <c r="B79" t="s">
+      <c r="C79" t="s">
         <v>538</v>
       </c>
-      <c r="C79" t="s">
+      <c r="D79" t="s">
         <v>539</v>
       </c>
-      <c r="D79" t="s">
+      <c r="E79" t="s">
         <v>540</v>
       </c>
-      <c r="E79" t="s">
+      <c r="F79" t="s">
         <v>541</v>
       </c>
-      <c r="F79" t="s">
+      <c r="G79" t="s">
         <v>542</v>
       </c>
-      <c r="G79" t="s">
-        <v>543</v>
-      </c>
       <c r="H79" t="s">
-        <v>1010</v>
+        <v>1009</v>
       </c>
       <c r="I79" t="s">
         <v>16</v>
@@ -6097,28 +6097,28 @@
     </row>
     <row r="80" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A80" t="s">
+        <v>543</v>
+      </c>
+      <c r="B80" t="s">
         <v>544</v>
       </c>
-      <c r="B80" t="s">
+      <c r="C80" t="s">
         <v>545</v>
       </c>
-      <c r="C80" t="s">
+      <c r="D80" t="s">
         <v>546</v>
       </c>
-      <c r="D80" t="s">
+      <c r="E80" t="s">
         <v>547</v>
       </c>
-      <c r="E80" t="s">
+      <c r="F80" t="s">
         <v>548</v>
       </c>
-      <c r="F80" t="s">
+      <c r="G80" t="s">
         <v>549</v>
       </c>
-      <c r="G80" t="s">
-        <v>550</v>
-      </c>
       <c r="H80" t="s">
-        <v>1015</v>
+        <v>1014</v>
       </c>
       <c r="I80" t="s">
         <v>7</v>
@@ -6129,28 +6129,28 @@
     </row>
     <row r="81" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A81" t="s">
+        <v>550</v>
+      </c>
+      <c r="B81" t="s">
         <v>551</v>
       </c>
-      <c r="B81" t="s">
+      <c r="C81" t="s">
         <v>552</v>
       </c>
-      <c r="C81" t="s">
+      <c r="D81" t="s">
         <v>553</v>
       </c>
-      <c r="D81" t="s">
+      <c r="E81" t="s">
         <v>554</v>
       </c>
-      <c r="E81" t="s">
+      <c r="F81" t="s">
         <v>555</v>
       </c>
-      <c r="F81" t="s">
-        <v>556</v>
-      </c>
       <c r="G81" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="H81" t="s">
-        <v>1016</v>
+        <v>1015</v>
       </c>
       <c r="I81" t="s">
         <v>16</v>
@@ -6161,28 +6161,28 @@
     </row>
     <row r="82" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A82" t="s">
+        <v>556</v>
+      </c>
+      <c r="B82" t="s">
         <v>557</v>
       </c>
-      <c r="B82" t="s">
+      <c r="C82" t="s">
         <v>558</v>
-      </c>
-      <c r="C82" t="s">
-        <v>559</v>
       </c>
       <c r="D82" t="s">
         <v>153</v>
       </c>
       <c r="E82" t="s">
+        <v>559</v>
+      </c>
+      <c r="F82" t="s">
         <v>560</v>
       </c>
-      <c r="F82" t="s">
+      <c r="G82" t="s">
         <v>561</v>
       </c>
-      <c r="G82" t="s">
-        <v>562</v>
-      </c>
       <c r="H82" t="s">
-        <v>1017</v>
+        <v>1016</v>
       </c>
       <c r="I82" t="s">
         <v>7</v>
@@ -6193,28 +6193,28 @@
     </row>
     <row r="83" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A83" t="s">
+        <v>562</v>
+      </c>
+      <c r="B83" t="s">
         <v>563</v>
       </c>
-      <c r="B83" t="s">
+      <c r="C83" t="s">
         <v>564</v>
       </c>
-      <c r="C83" t="s">
+      <c r="D83" t="s">
         <v>565</v>
       </c>
-      <c r="D83" t="s">
+      <c r="E83" t="s">
         <v>566</v>
       </c>
-      <c r="E83" t="s">
+      <c r="F83" t="s">
         <v>567</v>
       </c>
-      <c r="F83" t="s">
+      <c r="G83" t="s">
         <v>568</v>
       </c>
-      <c r="G83" t="s">
-        <v>569</v>
-      </c>
       <c r="H83" t="s">
-        <v>1010</v>
+        <v>1009</v>
       </c>
       <c r="I83" t="s">
         <v>7</v>
@@ -6225,28 +6225,28 @@
     </row>
     <row r="84" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A84" t="s">
+        <v>569</v>
+      </c>
+      <c r="B84" t="s">
         <v>570</v>
       </c>
-      <c r="B84" t="s">
+      <c r="C84" t="s">
         <v>571</v>
       </c>
-      <c r="C84" t="s">
+      <c r="D84" t="s">
         <v>572</v>
       </c>
-      <c r="D84" t="s">
+      <c r="E84" t="s">
         <v>573</v>
       </c>
-      <c r="E84" t="s">
+      <c r="F84" t="s">
         <v>574</v>
       </c>
-      <c r="F84" t="s">
+      <c r="G84" t="s">
         <v>575</v>
       </c>
-      <c r="G84" t="s">
-        <v>576</v>
-      </c>
       <c r="H84" t="s">
-        <v>1018</v>
+        <v>1017</v>
       </c>
       <c r="I84" t="s">
         <v>7</v>
@@ -6257,28 +6257,28 @@
     </row>
     <row r="85" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A85" t="s">
+        <v>576</v>
+      </c>
+      <c r="B85" t="s">
         <v>577</v>
       </c>
-      <c r="B85" t="s">
+      <c r="C85" t="s">
         <v>578</v>
       </c>
-      <c r="C85" t="s">
+      <c r="D85" t="s">
         <v>579</v>
       </c>
-      <c r="D85" t="s">
+      <c r="E85" t="s">
         <v>580</v>
       </c>
-      <c r="E85" t="s">
+      <c r="F85" t="s">
         <v>581</v>
       </c>
-      <c r="F85" t="s">
+      <c r="G85" t="s">
         <v>582</v>
       </c>
-      <c r="G85" t="s">
-        <v>583</v>
-      </c>
       <c r="H85" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
       <c r="I85" t="s">
         <v>7</v>
@@ -6289,28 +6289,28 @@
     </row>
     <row r="86" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A86" t="s">
+        <v>583</v>
+      </c>
+      <c r="B86" t="s">
         <v>584</v>
       </c>
-      <c r="B86" t="s">
+      <c r="C86" t="s">
         <v>585</v>
       </c>
-      <c r="C86" t="s">
+      <c r="D86" t="s">
         <v>586</v>
       </c>
-      <c r="D86" t="s">
+      <c r="E86" t="s">
         <v>587</v>
       </c>
-      <c r="E86" t="s">
+      <c r="F86" t="s">
         <v>588</v>
       </c>
-      <c r="F86" t="s">
+      <c r="G86" t="s">
         <v>589</v>
       </c>
-      <c r="G86" t="s">
-        <v>590</v>
-      </c>
       <c r="H86" t="s">
-        <v>1018</v>
+        <v>1017</v>
       </c>
       <c r="I86" t="s">
         <v>16</v>
@@ -6321,28 +6321,28 @@
     </row>
     <row r="87" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A87" t="s">
+        <v>590</v>
+      </c>
+      <c r="B87" t="s">
         <v>591</v>
       </c>
-      <c r="B87" t="s">
+      <c r="C87" t="s">
         <v>592</v>
       </c>
-      <c r="C87" t="s">
+      <c r="D87" t="s">
         <v>593</v>
       </c>
-      <c r="D87" t="s">
+      <c r="E87" t="s">
         <v>594</v>
       </c>
-      <c r="E87" t="s">
+      <c r="F87" t="s">
         <v>595</v>
       </c>
-      <c r="F87" t="s">
+      <c r="G87" t="s">
         <v>596</v>
       </c>
-      <c r="G87" t="s">
-        <v>597</v>
-      </c>
       <c r="H87" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
       <c r="I87" t="s">
         <v>16</v>
@@ -6353,63 +6353,63 @@
     </row>
     <row r="88" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A88" t="s">
+        <v>597</v>
+      </c>
+      <c r="B88" t="s">
         <v>598</v>
       </c>
-      <c r="B88" t="s">
+      <c r="C88" t="s">
         <v>599</v>
       </c>
-      <c r="C88" t="s">
+      <c r="D88" t="s">
         <v>600</v>
       </c>
-      <c r="D88" t="s">
+      <c r="E88" t="s">
         <v>601</v>
       </c>
-      <c r="E88" t="s">
+      <c r="F88" t="s">
         <v>602</v>
       </c>
-      <c r="F88" t="s">
+      <c r="G88" t="s">
         <v>603</v>
       </c>
-      <c r="G88" t="s">
+      <c r="H88" t="s">
+        <v>1017</v>
+      </c>
+      <c r="I88" t="s">
+        <v>16</v>
+      </c>
+      <c r="J88" t="s">
+        <v>1049</v>
+      </c>
+      <c r="K88" t="s">
         <v>604</v>
-      </c>
-      <c r="H88" t="s">
-        <v>1018</v>
-      </c>
-      <c r="I88" t="s">
-        <v>16</v>
-      </c>
-      <c r="J88" t="s">
-        <v>246</v>
-      </c>
-      <c r="K88" t="s">
-        <v>605</v>
       </c>
     </row>
     <row r="89" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A89" t="s">
+        <v>605</v>
+      </c>
+      <c r="B89" t="s">
         <v>606</v>
       </c>
-      <c r="B89" t="s">
+      <c r="C89" t="s">
         <v>607</v>
       </c>
-      <c r="C89" t="s">
+      <c r="D89" t="s">
         <v>608</v>
       </c>
-      <c r="D89" t="s">
+      <c r="E89" t="s">
         <v>609</v>
       </c>
-      <c r="E89" t="s">
+      <c r="F89" t="s">
         <v>610</v>
       </c>
-      <c r="F89" t="s">
+      <c r="G89" t="s">
         <v>611</v>
       </c>
-      <c r="G89" t="s">
-        <v>612</v>
-      </c>
       <c r="H89" t="s">
-        <v>983</v>
+        <v>982</v>
       </c>
       <c r="I89" t="s">
         <v>16</v>
@@ -6420,28 +6420,28 @@
     </row>
     <row r="90" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A90" t="s">
+        <v>612</v>
+      </c>
+      <c r="B90" t="s">
         <v>613</v>
       </c>
-      <c r="B90" t="s">
+      <c r="C90" t="s">
         <v>614</v>
       </c>
-      <c r="C90" t="s">
+      <c r="D90" t="s">
         <v>615</v>
       </c>
-      <c r="D90" t="s">
+      <c r="E90" t="s">
         <v>616</v>
       </c>
-      <c r="E90" t="s">
+      <c r="F90" t="s">
         <v>617</v>
       </c>
-      <c r="F90" t="s">
-        <v>618</v>
-      </c>
       <c r="G90" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="H90" t="s">
-        <v>983</v>
+        <v>982</v>
       </c>
       <c r="I90" t="s">
         <v>16</v>
@@ -6452,28 +6452,28 @@
     </row>
     <row r="91" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A91" t="s">
+        <v>618</v>
+      </c>
+      <c r="B91" t="s">
         <v>619</v>
       </c>
-      <c r="B91" t="s">
+      <c r="C91" t="s">
+        <v>456</v>
+      </c>
+      <c r="D91" t="s">
         <v>620</v>
       </c>
-      <c r="C91" t="s">
-        <v>457</v>
-      </c>
-      <c r="D91" t="s">
+      <c r="E91" t="s">
         <v>621</v>
       </c>
-      <c r="E91" t="s">
+      <c r="F91" t="s">
         <v>622</v>
       </c>
-      <c r="F91" t="s">
+      <c r="G91" t="s">
         <v>623</v>
       </c>
-      <c r="G91" t="s">
-        <v>624</v>
-      </c>
       <c r="H91" t="s">
-        <v>983</v>
+        <v>982</v>
       </c>
       <c r="I91" t="s">
         <v>7</v>
@@ -6484,28 +6484,28 @@
     </row>
     <row r="92" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A92" t="s">
+        <v>624</v>
+      </c>
+      <c r="B92" t="s">
         <v>625</v>
       </c>
-      <c r="B92" t="s">
+      <c r="C92" t="s">
         <v>626</v>
       </c>
-      <c r="C92" t="s">
+      <c r="D92" t="s">
         <v>627</v>
       </c>
-      <c r="D92" t="s">
+      <c r="E92" t="s">
         <v>628</v>
       </c>
-      <c r="E92" t="s">
+      <c r="F92" t="s">
         <v>629</v>
       </c>
-      <c r="F92" t="s">
+      <c r="G92" t="s">
         <v>630</v>
       </c>
-      <c r="G92" t="s">
-        <v>631</v>
-      </c>
       <c r="H92" t="s">
-        <v>1021</v>
+        <v>1020</v>
       </c>
       <c r="I92" t="s">
         <v>16</v>
@@ -6516,63 +6516,63 @@
     </row>
     <row r="93" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A93" t="s">
+        <v>631</v>
+      </c>
+      <c r="B93" t="s">
         <v>632</v>
       </c>
-      <c r="B93" t="s">
+      <c r="C93" t="s">
         <v>633</v>
       </c>
-      <c r="C93" t="s">
+      <c r="D93" t="s">
         <v>634</v>
       </c>
-      <c r="D93" t="s">
+      <c r="E93" t="s">
         <v>635</v>
       </c>
-      <c r="E93" t="s">
+      <c r="F93" t="s">
         <v>636</v>
       </c>
-      <c r="F93" t="s">
+      <c r="G93" t="s">
         <v>637</v>
       </c>
-      <c r="G93" t="s">
+      <c r="H93" t="s">
+        <v>979</v>
+      </c>
+      <c r="I93" t="s">
+        <v>16</v>
+      </c>
+      <c r="J93" t="s">
+        <v>1049</v>
+      </c>
+      <c r="K93" t="s">
         <v>638</v>
-      </c>
-      <c r="H93" t="s">
-        <v>980</v>
-      </c>
-      <c r="I93" t="s">
-        <v>16</v>
-      </c>
-      <c r="J93" t="s">
-        <v>246</v>
-      </c>
-      <c r="K93" t="s">
-        <v>639</v>
       </c>
     </row>
     <row r="94" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A94" t="s">
+        <v>639</v>
+      </c>
+      <c r="B94" t="s">
         <v>640</v>
       </c>
-      <c r="B94" t="s">
+      <c r="C94" t="s">
         <v>641</v>
       </c>
-      <c r="C94" t="s">
+      <c r="D94" t="s">
         <v>642</v>
       </c>
-      <c r="D94" t="s">
+      <c r="E94" t="s">
         <v>643</v>
       </c>
-      <c r="E94" t="s">
+      <c r="F94" t="s">
         <v>644</v>
       </c>
-      <c r="F94" t="s">
+      <c r="G94" t="s">
         <v>645</v>
       </c>
-      <c r="G94" t="s">
-        <v>646</v>
-      </c>
       <c r="H94" t="s">
-        <v>1022</v>
+        <v>1021</v>
       </c>
       <c r="I94" t="s">
         <v>16</v>
@@ -6583,28 +6583,28 @@
     </row>
     <row r="95" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A95" t="s">
+        <v>646</v>
+      </c>
+      <c r="B95" t="s">
         <v>647</v>
       </c>
-      <c r="B95" t="s">
+      <c r="C95" t="s">
         <v>648</v>
       </c>
-      <c r="C95" t="s">
+      <c r="D95" t="s">
         <v>649</v>
       </c>
-      <c r="D95" t="s">
+      <c r="E95" t="s">
         <v>650</v>
       </c>
-      <c r="E95" t="s">
+      <c r="F95" t="s">
         <v>651</v>
       </c>
-      <c r="F95" t="s">
+      <c r="G95" t="s">
         <v>652</v>
       </c>
-      <c r="G95" t="s">
-        <v>653</v>
-      </c>
       <c r="H95" t="s">
-        <v>1022</v>
+        <v>1021</v>
       </c>
       <c r="I95" t="s">
         <v>16</v>
@@ -6615,28 +6615,28 @@
     </row>
     <row r="96" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A96" t="s">
+        <v>653</v>
+      </c>
+      <c r="B96" t="s">
         <v>654</v>
       </c>
-      <c r="B96" t="s">
+      <c r="C96" t="s">
         <v>655</v>
       </c>
-      <c r="C96" t="s">
+      <c r="D96" t="s">
         <v>656</v>
       </c>
-      <c r="D96" t="s">
+      <c r="E96" t="s">
         <v>657</v>
       </c>
-      <c r="E96" t="s">
+      <c r="F96" t="s">
         <v>658</v>
       </c>
-      <c r="F96" t="s">
+      <c r="G96" t="s">
         <v>659</v>
       </c>
-      <c r="G96" t="s">
-        <v>660</v>
-      </c>
       <c r="H96" t="s">
-        <v>1022</v>
+        <v>1021</v>
       </c>
       <c r="I96" t="s">
         <v>16</v>
@@ -6647,28 +6647,28 @@
     </row>
     <row r="97" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A97" t="s">
+        <v>660</v>
+      </c>
+      <c r="B97" t="s">
         <v>661</v>
       </c>
-      <c r="B97" t="s">
+      <c r="C97" t="s">
         <v>662</v>
       </c>
-      <c r="C97" t="s">
+      <c r="D97" t="s">
         <v>663</v>
       </c>
-      <c r="D97" t="s">
+      <c r="E97" t="s">
         <v>664</v>
       </c>
-      <c r="E97" t="s">
+      <c r="F97" t="s">
         <v>665</v>
       </c>
-      <c r="F97" t="s">
+      <c r="G97" t="s">
         <v>666</v>
       </c>
-      <c r="G97" t="s">
-        <v>667</v>
-      </c>
       <c r="H97" t="s">
-        <v>1023</v>
+        <v>1022</v>
       </c>
       <c r="I97" t="s">
         <v>16</v>
@@ -6679,28 +6679,28 @@
     </row>
     <row r="98" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A98" t="s">
+        <v>667</v>
+      </c>
+      <c r="B98" t="s">
         <v>668</v>
       </c>
-      <c r="B98" t="s">
+      <c r="C98" t="s">
         <v>669</v>
       </c>
-      <c r="C98" t="s">
+      <c r="D98" t="s">
         <v>670</v>
       </c>
-      <c r="D98" t="s">
+      <c r="E98" t="s">
         <v>671</v>
       </c>
-      <c r="E98" t="s">
+      <c r="F98" t="s">
         <v>672</v>
       </c>
-      <c r="F98" t="s">
+      <c r="G98" t="s">
         <v>673</v>
       </c>
-      <c r="G98" t="s">
-        <v>674</v>
-      </c>
       <c r="H98" t="s">
-        <v>1001</v>
+        <v>1000</v>
       </c>
       <c r="I98" t="s">
         <v>7</v>
@@ -6711,28 +6711,28 @@
     </row>
     <row r="99" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A99" t="s">
+        <v>674</v>
+      </c>
+      <c r="B99" t="s">
         <v>675</v>
       </c>
-      <c r="B99" t="s">
+      <c r="C99" t="s">
         <v>676</v>
       </c>
-      <c r="C99" t="s">
+      <c r="D99" t="s">
         <v>677</v>
       </c>
-      <c r="D99" t="s">
+      <c r="E99" t="s">
         <v>678</v>
       </c>
-      <c r="E99" t="s">
+      <c r="F99" t="s">
         <v>679</v>
       </c>
-      <c r="F99" t="s">
+      <c r="G99" t="s">
         <v>680</v>
       </c>
-      <c r="G99" t="s">
-        <v>681</v>
-      </c>
       <c r="H99" t="s">
-        <v>1024</v>
+        <v>1023</v>
       </c>
       <c r="I99" t="s">
         <v>16</v>
@@ -6743,28 +6743,28 @@
     </row>
     <row r="100" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A100" t="s">
+        <v>681</v>
+      </c>
+      <c r="B100" t="s">
         <v>682</v>
       </c>
-      <c r="B100" t="s">
+      <c r="C100" t="s">
         <v>683</v>
       </c>
-      <c r="C100" t="s">
+      <c r="D100" t="s">
         <v>684</v>
       </c>
-      <c r="D100" t="s">
+      <c r="E100" t="s">
         <v>685</v>
       </c>
-      <c r="E100" t="s">
+      <c r="F100" t="s">
         <v>686</v>
       </c>
-      <c r="F100" t="s">
+      <c r="G100" t="s">
         <v>687</v>
       </c>
-      <c r="G100" t="s">
-        <v>688</v>
-      </c>
       <c r="H100" t="s">
-        <v>976</v>
+        <v>975</v>
       </c>
       <c r="I100" t="s">
         <v>7</v>
@@ -6775,28 +6775,28 @@
     </row>
     <row r="101" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A101" t="s">
+        <v>688</v>
+      </c>
+      <c r="B101" t="s">
         <v>689</v>
       </c>
-      <c r="B101" t="s">
+      <c r="C101" t="s">
         <v>690</v>
       </c>
-      <c r="C101" t="s">
+      <c r="D101" t="s">
         <v>691</v>
       </c>
-      <c r="D101" t="s">
+      <c r="E101" t="s">
         <v>692</v>
       </c>
-      <c r="E101" t="s">
+      <c r="F101" t="s">
         <v>693</v>
       </c>
-      <c r="F101" t="s">
+      <c r="G101" t="s">
         <v>694</v>
       </c>
-      <c r="G101" t="s">
-        <v>695</v>
-      </c>
       <c r="H101" t="s">
-        <v>995</v>
+        <v>994</v>
       </c>
       <c r="I101" t="s">
         <v>16</v>
@@ -6807,28 +6807,28 @@
     </row>
     <row r="102" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A102" t="s">
+        <v>695</v>
+      </c>
+      <c r="B102" t="s">
         <v>696</v>
       </c>
-      <c r="B102" t="s">
+      <c r="C102" t="s">
         <v>697</v>
       </c>
-      <c r="C102" t="s">
+      <c r="D102" t="s">
         <v>698</v>
       </c>
-      <c r="D102" t="s">
+      <c r="E102" t="s">
         <v>699</v>
       </c>
-      <c r="E102" t="s">
+      <c r="F102" t="s">
         <v>700</v>
       </c>
-      <c r="F102" t="s">
+      <c r="G102" t="s">
         <v>701</v>
       </c>
-      <c r="G102" t="s">
-        <v>702</v>
-      </c>
       <c r="H102" t="s">
-        <v>976</v>
+        <v>975</v>
       </c>
       <c r="I102" t="s">
         <v>16</v>
@@ -6839,28 +6839,28 @@
     </row>
     <row r="103" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A103" t="s">
+        <v>702</v>
+      </c>
+      <c r="B103" t="s">
         <v>703</v>
       </c>
-      <c r="B103" t="s">
+      <c r="C103" t="s">
         <v>704</v>
       </c>
-      <c r="C103" t="s">
+      <c r="D103" t="s">
         <v>705</v>
       </c>
-      <c r="D103" t="s">
+      <c r="E103" t="s">
         <v>706</v>
       </c>
-      <c r="E103" t="s">
+      <c r="F103" t="s">
         <v>707</v>
       </c>
-      <c r="F103" t="s">
+      <c r="G103" t="s">
         <v>708</v>
       </c>
-      <c r="G103" t="s">
-        <v>709</v>
-      </c>
       <c r="H103" t="s">
-        <v>976</v>
+        <v>975</v>
       </c>
       <c r="I103" t="s">
         <v>16</v>
@@ -6871,28 +6871,28 @@
     </row>
     <row r="104" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A104" t="s">
+        <v>709</v>
+      </c>
+      <c r="B104" t="s">
         <v>710</v>
       </c>
-      <c r="B104" t="s">
+      <c r="C104" t="s">
         <v>711</v>
       </c>
-      <c r="C104" t="s">
+      <c r="D104" t="s">
         <v>712</v>
       </c>
-      <c r="D104" t="s">
+      <c r="E104" t="s">
         <v>713</v>
       </c>
-      <c r="E104" t="s">
+      <c r="F104" t="s">
         <v>714</v>
       </c>
-      <c r="F104" t="s">
+      <c r="G104" t="s">
         <v>715</v>
       </c>
-      <c r="G104" t="s">
-        <v>716</v>
-      </c>
       <c r="H104" t="s">
-        <v>1025</v>
+        <v>1024</v>
       </c>
       <c r="I104" t="s">
         <v>7</v>
@@ -6903,28 +6903,28 @@
     </row>
     <row r="105" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A105" t="s">
+        <v>716</v>
+      </c>
+      <c r="B105" t="s">
         <v>717</v>
       </c>
-      <c r="B105" t="s">
+      <c r="C105" t="s">
         <v>718</v>
       </c>
-      <c r="C105" t="s">
+      <c r="D105" t="s">
         <v>719</v>
       </c>
-      <c r="D105" t="s">
+      <c r="E105" t="s">
         <v>720</v>
       </c>
-      <c r="E105" t="s">
+      <c r="F105" t="s">
         <v>721</v>
       </c>
-      <c r="F105" t="s">
+      <c r="G105" t="s">
         <v>722</v>
       </c>
-      <c r="G105" t="s">
-        <v>723</v>
-      </c>
       <c r="H105" t="s">
-        <v>1026</v>
+        <v>1025</v>
       </c>
       <c r="I105" t="s">
         <v>7</v>
@@ -6935,28 +6935,28 @@
     </row>
     <row r="106" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A106" t="s">
+        <v>723</v>
+      </c>
+      <c r="B106" t="s">
         <v>724</v>
       </c>
-      <c r="B106" t="s">
+      <c r="C106" t="s">
         <v>725</v>
       </c>
-      <c r="C106" t="s">
+      <c r="D106" t="s">
         <v>726</v>
       </c>
-      <c r="D106" t="s">
+      <c r="E106" t="s">
         <v>727</v>
       </c>
-      <c r="E106" t="s">
+      <c r="F106" t="s">
         <v>728</v>
       </c>
-      <c r="F106" t="s">
+      <c r="G106" t="s">
         <v>729</v>
       </c>
-      <c r="G106" t="s">
-        <v>730</v>
-      </c>
       <c r="H106" t="s">
-        <v>978</v>
+        <v>977</v>
       </c>
       <c r="I106" t="s">
         <v>7</v>
@@ -6967,28 +6967,28 @@
     </row>
     <row r="107" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A107" t="s">
+        <v>730</v>
+      </c>
+      <c r="B107" t="s">
         <v>731</v>
       </c>
-      <c r="B107" t="s">
+      <c r="C107" t="s">
         <v>732</v>
       </c>
-      <c r="C107" t="s">
+      <c r="D107" t="s">
         <v>733</v>
       </c>
-      <c r="D107" t="s">
+      <c r="E107" t="s">
         <v>734</v>
       </c>
-      <c r="E107" t="s">
+      <c r="F107" t="s">
         <v>735</v>
       </c>
-      <c r="F107" t="s">
+      <c r="G107" t="s">
         <v>736</v>
       </c>
-      <c r="G107" t="s">
-        <v>737</v>
-      </c>
       <c r="H107" t="s">
-        <v>1027</v>
+        <v>1026</v>
       </c>
       <c r="I107" t="s">
         <v>7</v>
@@ -6999,28 +6999,28 @@
     </row>
     <row r="108" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A108" t="s">
+        <v>737</v>
+      </c>
+      <c r="B108" t="s">
         <v>738</v>
       </c>
-      <c r="B108" t="s">
+      <c r="C108" t="s">
         <v>739</v>
       </c>
-      <c r="C108" t="s">
+      <c r="D108" t="s">
         <v>740</v>
       </c>
-      <c r="D108" t="s">
+      <c r="E108" t="s">
         <v>741</v>
       </c>
-      <c r="E108" t="s">
+      <c r="F108" t="s">
         <v>742</v>
       </c>
-      <c r="F108" t="s">
+      <c r="G108" t="s">
         <v>743</v>
       </c>
-      <c r="G108" t="s">
-        <v>744</v>
-      </c>
       <c r="H108" t="s">
-        <v>1028</v>
+        <v>1027</v>
       </c>
       <c r="I108" t="s">
         <v>7</v>
@@ -7031,28 +7031,28 @@
     </row>
     <row r="109" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A109" t="s">
+        <v>744</v>
+      </c>
+      <c r="B109" t="s">
         <v>745</v>
       </c>
-      <c r="B109" t="s">
+      <c r="C109" t="s">
         <v>746</v>
       </c>
-      <c r="C109" t="s">
+      <c r="D109" t="s">
         <v>747</v>
       </c>
-      <c r="D109" t="s">
+      <c r="E109" t="s">
         <v>748</v>
       </c>
-      <c r="E109" t="s">
+      <c r="F109" t="s">
         <v>749</v>
       </c>
-      <c r="F109" t="s">
+      <c r="G109" t="s">
         <v>750</v>
       </c>
-      <c r="G109" t="s">
-        <v>751</v>
-      </c>
       <c r="H109" t="s">
-        <v>1029</v>
+        <v>1028</v>
       </c>
       <c r="I109" t="s">
         <v>7</v>
@@ -7063,28 +7063,28 @@
     </row>
     <row r="110" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A110" t="s">
+        <v>751</v>
+      </c>
+      <c r="B110" t="s">
         <v>752</v>
       </c>
-      <c r="B110" t="s">
+      <c r="C110" t="s">
         <v>753</v>
       </c>
-      <c r="C110" t="s">
+      <c r="D110" t="s">
         <v>754</v>
       </c>
-      <c r="D110" t="s">
+      <c r="E110" t="s">
         <v>755</v>
       </c>
-      <c r="E110" t="s">
+      <c r="F110" t="s">
         <v>756</v>
       </c>
-      <c r="F110" t="s">
+      <c r="G110" t="s">
         <v>757</v>
       </c>
-      <c r="G110" t="s">
-        <v>758</v>
-      </c>
       <c r="H110" t="s">
-        <v>994</v>
+        <v>993</v>
       </c>
       <c r="I110" t="s">
         <v>16</v>
@@ -7095,28 +7095,28 @@
     </row>
     <row r="111" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A111" t="s">
+        <v>758</v>
+      </c>
+      <c r="B111" t="s">
         <v>759</v>
       </c>
-      <c r="B111" t="s">
+      <c r="C111" t="s">
         <v>760</v>
       </c>
-      <c r="C111" t="s">
+      <c r="D111" t="s">
         <v>761</v>
       </c>
-      <c r="D111" t="s">
+      <c r="E111" t="s">
         <v>762</v>
       </c>
-      <c r="E111" t="s">
+      <c r="F111" t="s">
         <v>763</v>
       </c>
-      <c r="F111" t="s">
-        <v>764</v>
-      </c>
       <c r="G111" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="H111" t="s">
-        <v>994</v>
+        <v>993</v>
       </c>
       <c r="I111" t="s">
         <v>7</v>
@@ -7127,28 +7127,28 @@
     </row>
     <row r="112" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A112" t="s">
+        <v>764</v>
+      </c>
+      <c r="B112" t="s">
         <v>765</v>
       </c>
-      <c r="B112" t="s">
+      <c r="C112" t="s">
         <v>766</v>
       </c>
-      <c r="C112" t="s">
+      <c r="D112" t="s">
         <v>767</v>
       </c>
-      <c r="D112" t="s">
+      <c r="E112" t="s">
         <v>768</v>
       </c>
-      <c r="E112" t="s">
+      <c r="F112" t="s">
         <v>769</v>
       </c>
-      <c r="F112" t="s">
+      <c r="G112" t="s">
         <v>770</v>
       </c>
-      <c r="G112" t="s">
-        <v>771</v>
-      </c>
       <c r="H112" t="s">
-        <v>1030</v>
+        <v>1029</v>
       </c>
       <c r="I112" t="s">
         <v>16</v>
@@ -7159,98 +7159,98 @@
     </row>
     <row r="113" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A113" t="s">
+        <v>771</v>
+      </c>
+      <c r="B113" t="s">
         <v>772</v>
       </c>
-      <c r="B113" t="s">
+      <c r="C113" t="s">
         <v>773</v>
       </c>
-      <c r="C113" t="s">
+      <c r="D113" t="s">
         <v>774</v>
       </c>
-      <c r="D113" t="s">
+      <c r="E113" t="s">
         <v>775</v>
       </c>
-      <c r="E113" t="s">
+      <c r="F113" t="s">
         <v>776</v>
       </c>
-      <c r="F113" t="s">
+      <c r="G113" t="s">
         <v>777</v>
       </c>
-      <c r="G113" t="s">
-        <v>778</v>
-      </c>
       <c r="H113" t="s">
-        <v>1031</v>
+        <v>1030</v>
       </c>
       <c r="I113" t="s">
         <v>16</v>
       </c>
       <c r="J113" t="s">
-        <v>246</v>
+        <v>1049</v>
       </c>
       <c r="K113" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
     </row>
     <row r="114" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A114" t="s">
+        <v>778</v>
+      </c>
+      <c r="B114" t="s">
         <v>779</v>
       </c>
-      <c r="B114" t="s">
+      <c r="C114" t="s">
         <v>780</v>
       </c>
-      <c r="C114" t="s">
+      <c r="D114" t="s">
         <v>781</v>
       </c>
-      <c r="D114" t="s">
+      <c r="E114" t="s">
         <v>782</v>
       </c>
-      <c r="E114" t="s">
+      <c r="F114" t="s">
         <v>783</v>
       </c>
-      <c r="F114" t="s">
+      <c r="G114" t="s">
         <v>784</v>
       </c>
-      <c r="G114" t="s">
+      <c r="H114" t="s">
+        <v>1031</v>
+      </c>
+      <c r="I114" t="s">
+        <v>16</v>
+      </c>
+      <c r="J114" t="s">
+        <v>1049</v>
+      </c>
+      <c r="K114" t="s">
         <v>785</v>
-      </c>
-      <c r="H114" t="s">
-        <v>1032</v>
-      </c>
-      <c r="I114" t="s">
-        <v>16</v>
-      </c>
-      <c r="J114" t="s">
-        <v>246</v>
-      </c>
-      <c r="K114" t="s">
-        <v>786</v>
       </c>
     </row>
     <row r="115" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A115" t="s">
+        <v>786</v>
+      </c>
+      <c r="B115" t="s">
         <v>787</v>
       </c>
-      <c r="B115" t="s">
+      <c r="C115" t="s">
         <v>788</v>
       </c>
-      <c r="C115" t="s">
+      <c r="D115" t="s">
         <v>789</v>
       </c>
-      <c r="D115" t="s">
+      <c r="E115" t="s">
         <v>790</v>
       </c>
-      <c r="E115" t="s">
+      <c r="F115" t="s">
         <v>791</v>
       </c>
-      <c r="F115" t="s">
+      <c r="G115" t="s">
         <v>792</v>
       </c>
-      <c r="G115" t="s">
-        <v>793</v>
-      </c>
       <c r="H115" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
       <c r="I115" t="s">
         <v>16</v>
@@ -7261,28 +7261,28 @@
     </row>
     <row r="116" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A116" t="s">
+        <v>793</v>
+      </c>
+      <c r="B116" t="s">
         <v>794</v>
       </c>
-      <c r="B116" t="s">
+      <c r="C116" t="s">
         <v>795</v>
       </c>
-      <c r="C116" t="s">
+      <c r="D116" t="s">
         <v>796</v>
       </c>
-      <c r="D116" t="s">
+      <c r="E116" t="s">
         <v>797</v>
       </c>
-      <c r="E116" t="s">
+      <c r="F116" t="s">
         <v>798</v>
       </c>
-      <c r="F116" t="s">
+      <c r="G116" t="s">
         <v>799</v>
       </c>
-      <c r="G116" t="s">
-        <v>800</v>
-      </c>
       <c r="H116" t="s">
-        <v>1033</v>
+        <v>1032</v>
       </c>
       <c r="I116" t="s">
         <v>16</v>
@@ -7293,28 +7293,28 @@
     </row>
     <row r="117" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A117" t="s">
+        <v>800</v>
+      </c>
+      <c r="B117" t="s">
         <v>801</v>
       </c>
-      <c r="B117" t="s">
+      <c r="C117" t="s">
         <v>802</v>
       </c>
-      <c r="C117" t="s">
+      <c r="D117" t="s">
         <v>803</v>
       </c>
-      <c r="D117" t="s">
+      <c r="E117" t="s">
         <v>804</v>
       </c>
-      <c r="E117" t="s">
+      <c r="F117" t="s">
+        <v>341</v>
+      </c>
+      <c r="G117" t="s">
         <v>805</v>
       </c>
-      <c r="F117" t="s">
-        <v>342</v>
-      </c>
-      <c r="G117" t="s">
-        <v>806</v>
-      </c>
       <c r="H117" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
       <c r="I117" t="s">
         <v>16</v>
@@ -7325,28 +7325,28 @@
     </row>
     <row r="118" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A118" t="s">
+        <v>806</v>
+      </c>
+      <c r="B118" t="s">
         <v>807</v>
       </c>
-      <c r="B118" t="s">
+      <c r="C118" t="s">
         <v>808</v>
       </c>
-      <c r="C118" t="s">
+      <c r="D118" t="s">
         <v>809</v>
       </c>
-      <c r="D118" t="s">
+      <c r="E118" t="s">
         <v>810</v>
       </c>
-      <c r="E118" t="s">
+      <c r="F118" t="s">
         <v>811</v>
       </c>
-      <c r="F118" t="s">
+      <c r="G118" t="s">
         <v>812</v>
       </c>
-      <c r="G118" t="s">
-        <v>813</v>
-      </c>
       <c r="H118" t="s">
-        <v>1034</v>
+        <v>1033</v>
       </c>
       <c r="I118" t="s">
         <v>16</v>
@@ -7357,28 +7357,28 @@
     </row>
     <row r="119" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A119" t="s">
+        <v>813</v>
+      </c>
+      <c r="B119" t="s">
         <v>814</v>
       </c>
-      <c r="B119" t="s">
+      <c r="C119" t="s">
         <v>815</v>
       </c>
-      <c r="C119" t="s">
+      <c r="D119" t="s">
         <v>816</v>
       </c>
-      <c r="D119" t="s">
+      <c r="E119" t="s">
         <v>817</v>
       </c>
-      <c r="E119" t="s">
+      <c r="F119" t="s">
         <v>818</v>
       </c>
-      <c r="F119" t="s">
+      <c r="G119" t="s">
         <v>819</v>
       </c>
-      <c r="G119" t="s">
-        <v>820</v>
-      </c>
       <c r="H119" t="s">
-        <v>1035</v>
+        <v>1034</v>
       </c>
       <c r="I119" t="s">
         <v>16</v>
@@ -7389,28 +7389,28 @@
     </row>
     <row r="120" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A120" t="s">
+        <v>820</v>
+      </c>
+      <c r="B120" t="s">
         <v>821</v>
       </c>
-      <c r="B120" t="s">
+      <c r="C120" t="s">
         <v>822</v>
       </c>
-      <c r="C120" t="s">
+      <c r="D120" t="s">
         <v>823</v>
       </c>
-      <c r="D120" t="s">
+      <c r="E120" t="s">
         <v>824</v>
       </c>
-      <c r="E120" t="s">
+      <c r="F120" t="s">
         <v>825</v>
       </c>
-      <c r="F120" t="s">
+      <c r="G120" t="s">
         <v>826</v>
       </c>
-      <c r="G120" t="s">
-        <v>827</v>
-      </c>
       <c r="H120" t="s">
-        <v>997</v>
+        <v>996</v>
       </c>
       <c r="I120" t="s">
         <v>16</v>
@@ -7421,28 +7421,28 @@
     </row>
     <row r="121" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A121" t="s">
+        <v>827</v>
+      </c>
+      <c r="B121" t="s">
         <v>828</v>
       </c>
-      <c r="B121" t="s">
+      <c r="C121" t="s">
         <v>829</v>
       </c>
-      <c r="C121" t="s">
+      <c r="D121" t="s">
         <v>830</v>
       </c>
-      <c r="D121" t="s">
+      <c r="E121" t="s">
         <v>831</v>
       </c>
-      <c r="E121" t="s">
+      <c r="F121" t="s">
         <v>832</v>
       </c>
-      <c r="F121" t="s">
+      <c r="G121" t="s">
         <v>833</v>
       </c>
-      <c r="G121" t="s">
-        <v>834</v>
-      </c>
       <c r="H121" t="s">
-        <v>1021</v>
+        <v>1020</v>
       </c>
       <c r="I121" t="s">
         <v>16</v>
@@ -7453,28 +7453,28 @@
     </row>
     <row r="122" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A122" t="s">
+        <v>834</v>
+      </c>
+      <c r="B122" t="s">
         <v>835</v>
       </c>
-      <c r="B122" t="s">
+      <c r="C122" t="s">
+        <v>281</v>
+      </c>
+      <c r="D122" t="s">
+        <v>280</v>
+      </c>
+      <c r="E122" t="s">
+        <v>278</v>
+      </c>
+      <c r="F122" t="s">
+        <v>277</v>
+      </c>
+      <c r="G122" t="s">
         <v>836</v>
       </c>
-      <c r="C122" t="s">
-        <v>282</v>
-      </c>
-      <c r="D122" t="s">
-        <v>281</v>
-      </c>
-      <c r="E122" t="s">
-        <v>279</v>
-      </c>
-      <c r="F122" t="s">
-        <v>278</v>
-      </c>
-      <c r="G122" t="s">
-        <v>837</v>
-      </c>
       <c r="H122" t="s">
-        <v>1036</v>
+        <v>1035</v>
       </c>
       <c r="I122" t="s">
         <v>16</v>
@@ -7485,28 +7485,28 @@
     </row>
     <row r="123" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A123" t="s">
+        <v>837</v>
+      </c>
+      <c r="B123" t="s">
         <v>838</v>
       </c>
-      <c r="B123" t="s">
+      <c r="C123" t="s">
         <v>839</v>
       </c>
-      <c r="C123" t="s">
+      <c r="D123" t="s">
         <v>840</v>
       </c>
-      <c r="D123" t="s">
+      <c r="E123" t="s">
         <v>841</v>
       </c>
-      <c r="E123" t="s">
+      <c r="F123" t="s">
         <v>842</v>
       </c>
-      <c r="F123" t="s">
+      <c r="G123" t="s">
         <v>843</v>
       </c>
-      <c r="G123" t="s">
-        <v>844</v>
-      </c>
       <c r="H123" t="s">
-        <v>1037</v>
+        <v>1036</v>
       </c>
       <c r="I123" t="s">
         <v>16</v>
@@ -7517,28 +7517,28 @@
     </row>
     <row r="124" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A124" t="s">
+        <v>844</v>
+      </c>
+      <c r="B124" t="s">
         <v>845</v>
       </c>
-      <c r="B124" t="s">
+      <c r="C124" t="s">
         <v>846</v>
       </c>
-      <c r="C124" t="s">
+      <c r="D124" t="s">
         <v>847</v>
       </c>
-      <c r="D124" t="s">
+      <c r="E124" t="s">
+        <v>419</v>
+      </c>
+      <c r="F124" t="s">
         <v>848</v>
       </c>
-      <c r="E124" t="s">
-        <v>420</v>
-      </c>
-      <c r="F124" t="s">
+      <c r="G124" t="s">
         <v>849</v>
       </c>
-      <c r="G124" t="s">
-        <v>850</v>
-      </c>
       <c r="H124" t="s">
-        <v>977</v>
+        <v>976</v>
       </c>
       <c r="I124" t="s">
         <v>16</v>
@@ -7549,28 +7549,28 @@
     </row>
     <row r="125" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A125" t="s">
+        <v>850</v>
+      </c>
+      <c r="B125" t="s">
         <v>851</v>
       </c>
-      <c r="B125" t="s">
+      <c r="C125" t="s">
         <v>852</v>
       </c>
-      <c r="C125" t="s">
+      <c r="D125" t="s">
         <v>853</v>
       </c>
-      <c r="D125" t="s">
+      <c r="E125" t="s">
         <v>854</v>
       </c>
-      <c r="E125" t="s">
+      <c r="F125" t="s">
         <v>855</v>
       </c>
-      <c r="F125" t="s">
+      <c r="G125" t="s">
         <v>856</v>
       </c>
-      <c r="G125" t="s">
-        <v>857</v>
-      </c>
       <c r="H125" t="s">
-        <v>977</v>
+        <v>976</v>
       </c>
       <c r="I125" t="s">
         <v>16</v>
@@ -7581,28 +7581,28 @@
     </row>
     <row r="126" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A126" t="s">
+        <v>857</v>
+      </c>
+      <c r="B126" t="s">
         <v>858</v>
       </c>
-      <c r="B126" t="s">
+      <c r="C126" t="s">
         <v>859</v>
       </c>
-      <c r="C126" t="s">
+      <c r="D126" t="s">
         <v>860</v>
       </c>
-      <c r="D126" t="s">
+      <c r="E126" t="s">
         <v>861</v>
       </c>
-      <c r="E126" t="s">
+      <c r="F126" t="s">
         <v>862</v>
       </c>
-      <c r="F126" t="s">
+      <c r="G126" t="s">
         <v>863</v>
       </c>
-      <c r="G126" t="s">
-        <v>864</v>
-      </c>
       <c r="H126" t="s">
-        <v>1038</v>
+        <v>1037</v>
       </c>
       <c r="I126" t="s">
         <v>7</v>
@@ -7613,28 +7613,28 @@
     </row>
     <row r="127" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A127" t="s">
+        <v>864</v>
+      </c>
+      <c r="B127" t="s">
         <v>865</v>
       </c>
-      <c r="B127" t="s">
+      <c r="C127" t="s">
         <v>866</v>
       </c>
-      <c r="C127" t="s">
+      <c r="D127" t="s">
         <v>867</v>
       </c>
-      <c r="D127" t="s">
+      <c r="E127" t="s">
         <v>868</v>
       </c>
-      <c r="E127" t="s">
+      <c r="F127" t="s">
         <v>869</v>
       </c>
-      <c r="F127" t="s">
+      <c r="G127" t="s">
         <v>870</v>
       </c>
-      <c r="G127" t="s">
-        <v>871</v>
-      </c>
       <c r="H127" t="s">
-        <v>1018</v>
+        <v>1017</v>
       </c>
       <c r="I127" t="s">
         <v>16</v>
@@ -7645,28 +7645,28 @@
     </row>
     <row r="128" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A128" t="s">
+        <v>871</v>
+      </c>
+      <c r="B128" t="s">
         <v>872</v>
       </c>
-      <c r="B128" t="s">
+      <c r="C128" t="s">
         <v>873</v>
       </c>
-      <c r="C128" t="s">
+      <c r="D128" t="s">
         <v>874</v>
       </c>
-      <c r="D128" t="s">
+      <c r="E128" t="s">
         <v>875</v>
       </c>
-      <c r="E128" t="s">
+      <c r="F128" t="s">
         <v>876</v>
       </c>
-      <c r="F128" t="s">
+      <c r="G128" t="s">
         <v>877</v>
       </c>
-      <c r="G128" t="s">
-        <v>878</v>
-      </c>
       <c r="H128" t="s">
-        <v>975</v>
+        <v>974</v>
       </c>
       <c r="I128" t="s">
         <v>16</v>
@@ -7677,28 +7677,28 @@
     </row>
     <row r="129" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A129" t="s">
+        <v>878</v>
+      </c>
+      <c r="B129" t="s">
         <v>879</v>
       </c>
-      <c r="B129" t="s">
+      <c r="C129" t="s">
         <v>880</v>
       </c>
-      <c r="C129" t="s">
+      <c r="D129" t="s">
         <v>881</v>
       </c>
-      <c r="D129" t="s">
+      <c r="E129" t="s">
         <v>882</v>
       </c>
-      <c r="E129" t="s">
+      <c r="F129" t="s">
         <v>883</v>
       </c>
-      <c r="F129" t="s">
-        <v>884</v>
-      </c>
       <c r="G129" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="H129" t="s">
-        <v>1026</v>
+        <v>1025</v>
       </c>
       <c r="I129" t="s">
         <v>16</v>
@@ -7709,28 +7709,28 @@
     </row>
     <row r="130" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A130" t="s">
+        <v>884</v>
+      </c>
+      <c r="B130" t="s">
         <v>885</v>
       </c>
-      <c r="B130" t="s">
+      <c r="C130" t="s">
         <v>886</v>
       </c>
-      <c r="C130" t="s">
+      <c r="D130" t="s">
         <v>887</v>
       </c>
-      <c r="D130" t="s">
+      <c r="E130" t="s">
         <v>888</v>
       </c>
-      <c r="E130" t="s">
+      <c r="F130" t="s">
         <v>889</v>
       </c>
-      <c r="F130" t="s">
+      <c r="G130" t="s">
         <v>890</v>
       </c>
-      <c r="G130" t="s">
-        <v>891</v>
-      </c>
       <c r="H130" t="s">
-        <v>992</v>
+        <v>991</v>
       </c>
       <c r="I130" t="s">
         <v>7</v>
@@ -7741,28 +7741,28 @@
     </row>
     <row r="131" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A131" t="s">
+        <v>891</v>
+      </c>
+      <c r="B131" t="s">
         <v>892</v>
       </c>
-      <c r="B131" t="s">
+      <c r="C131" t="s">
         <v>893</v>
       </c>
-      <c r="C131" t="s">
+      <c r="D131" t="s">
         <v>894</v>
       </c>
-      <c r="D131" t="s">
+      <c r="E131" t="s">
         <v>895</v>
       </c>
-      <c r="E131" t="s">
+      <c r="F131" t="s">
         <v>896</v>
       </c>
-      <c r="F131" t="s">
+      <c r="G131" t="s">
         <v>897</v>
       </c>
-      <c r="G131" t="s">
-        <v>898</v>
-      </c>
       <c r="H131" t="s">
-        <v>1039</v>
+        <v>1038</v>
       </c>
       <c r="I131" t="s">
         <v>7</v>
@@ -7773,28 +7773,28 @@
     </row>
     <row r="132" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A132" t="s">
+        <v>898</v>
+      </c>
+      <c r="B132" t="s">
         <v>899</v>
       </c>
-      <c r="B132" t="s">
+      <c r="C132" t="s">
         <v>900</v>
       </c>
-      <c r="C132" t="s">
+      <c r="D132" t="s">
         <v>901</v>
       </c>
-      <c r="D132" t="s">
+      <c r="E132" t="s">
         <v>902</v>
       </c>
-      <c r="E132" t="s">
+      <c r="F132" t="s">
         <v>903</v>
       </c>
-      <c r="F132" t="s">
+      <c r="G132" t="s">
         <v>904</v>
       </c>
-      <c r="G132" t="s">
-        <v>905</v>
-      </c>
       <c r="H132" t="s">
-        <v>1040</v>
+        <v>1039</v>
       </c>
       <c r="I132" t="s">
         <v>7</v>
@@ -7805,28 +7805,28 @@
     </row>
     <row r="133" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A133" t="s">
+        <v>905</v>
+      </c>
+      <c r="B133" t="s">
         <v>906</v>
       </c>
-      <c r="B133" t="s">
+      <c r="C133" t="s">
         <v>907</v>
       </c>
-      <c r="C133" t="s">
+      <c r="D133" t="s">
         <v>908</v>
       </c>
-      <c r="D133" t="s">
+      <c r="E133" t="s">
         <v>909</v>
       </c>
-      <c r="E133" t="s">
+      <c r="F133" t="s">
         <v>910</v>
       </c>
-      <c r="F133" t="s">
+      <c r="G133" t="s">
         <v>911</v>
       </c>
-      <c r="G133" t="s">
-        <v>912</v>
-      </c>
       <c r="H133" t="s">
-        <v>1041</v>
+        <v>1040</v>
       </c>
       <c r="I133" t="s">
         <v>7</v>
@@ -7837,28 +7837,28 @@
     </row>
     <row r="134" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A134" t="s">
+        <v>912</v>
+      </c>
+      <c r="B134" t="s">
         <v>913</v>
       </c>
-      <c r="B134" t="s">
+      <c r="C134" t="s">
         <v>914</v>
       </c>
-      <c r="C134" t="s">
+      <c r="D134" t="s">
         <v>915</v>
       </c>
-      <c r="D134" t="s">
+      <c r="E134" t="s">
         <v>916</v>
       </c>
-      <c r="E134" t="s">
+      <c r="F134" t="s">
         <v>917</v>
       </c>
-      <c r="F134" t="s">
+      <c r="G134" t="s">
         <v>918</v>
       </c>
-      <c r="G134" t="s">
-        <v>919</v>
-      </c>
       <c r="H134" t="s">
-        <v>1042</v>
+        <v>1041</v>
       </c>
       <c r="I134" t="s">
         <v>16</v>
@@ -7869,28 +7869,28 @@
     </row>
     <row r="135" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A135" t="s">
+        <v>919</v>
+      </c>
+      <c r="B135" t="s">
         <v>920</v>
       </c>
-      <c r="B135" t="s">
+      <c r="C135" t="s">
         <v>921</v>
       </c>
-      <c r="C135" t="s">
+      <c r="D135" t="s">
         <v>922</v>
       </c>
-      <c r="D135" t="s">
+      <c r="E135" t="s">
         <v>923</v>
       </c>
-      <c r="E135" t="s">
+      <c r="F135" t="s">
         <v>924</v>
       </c>
-      <c r="F135" t="s">
+      <c r="G135" t="s">
         <v>925</v>
       </c>
-      <c r="G135" t="s">
-        <v>926</v>
-      </c>
       <c r="H135" t="s">
-        <v>996</v>
+        <v>995</v>
       </c>
       <c r="I135" t="s">
         <v>7</v>
@@ -7901,28 +7901,28 @@
     </row>
     <row r="136" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A136" t="s">
+        <v>926</v>
+      </c>
+      <c r="B136" t="s">
         <v>927</v>
       </c>
-      <c r="B136" t="s">
+      <c r="C136" t="s">
         <v>928</v>
       </c>
-      <c r="C136" t="s">
+      <c r="D136" t="s">
         <v>929</v>
       </c>
-      <c r="D136" t="s">
+      <c r="E136" t="s">
         <v>930</v>
       </c>
-      <c r="E136" t="s">
+      <c r="F136" t="s">
+        <v>355</v>
+      </c>
+      <c r="G136" t="s">
         <v>931</v>
       </c>
-      <c r="F136" t="s">
-        <v>356</v>
-      </c>
-      <c r="G136" t="s">
-        <v>932</v>
-      </c>
       <c r="H136" t="s">
-        <v>996</v>
+        <v>995</v>
       </c>
       <c r="I136" t="s">
         <v>7</v>
@@ -7933,28 +7933,28 @@
     </row>
     <row r="137" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A137" t="s">
+        <v>932</v>
+      </c>
+      <c r="B137" t="s">
         <v>933</v>
-      </c>
-      <c r="B137" t="s">
-        <v>934</v>
       </c>
       <c r="C137" t="s">
         <v>14</v>
       </c>
       <c r="D137" t="s">
+        <v>934</v>
+      </c>
+      <c r="E137" t="s">
         <v>935</v>
       </c>
-      <c r="E137" t="s">
+      <c r="F137" t="s">
         <v>936</v>
       </c>
-      <c r="F137" t="s">
+      <c r="G137" t="s">
         <v>937</v>
       </c>
-      <c r="G137" t="s">
-        <v>938</v>
-      </c>
       <c r="H137" t="s">
-        <v>1043</v>
+        <v>1042</v>
       </c>
       <c r="I137" t="s">
         <v>16</v>
@@ -7965,28 +7965,28 @@
     </row>
     <row r="138" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A138" t="s">
+        <v>938</v>
+      </c>
+      <c r="B138" t="s">
         <v>939</v>
       </c>
-      <c r="B138" t="s">
+      <c r="C138" t="s">
         <v>940</v>
       </c>
-      <c r="C138" t="s">
+      <c r="D138" t="s">
         <v>941</v>
       </c>
-      <c r="D138" t="s">
+      <c r="E138" t="s">
         <v>942</v>
       </c>
-      <c r="E138" t="s">
+      <c r="F138" t="s">
         <v>943</v>
       </c>
-      <c r="F138" t="s">
+      <c r="G138" t="s">
         <v>944</v>
       </c>
-      <c r="G138" t="s">
-        <v>945</v>
-      </c>
       <c r="H138" t="s">
-        <v>1044</v>
+        <v>1043</v>
       </c>
       <c r="I138" t="s">
         <v>7</v>
@@ -7997,28 +7997,28 @@
     </row>
     <row r="139" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A139" t="s">
+        <v>945</v>
+      </c>
+      <c r="B139" t="s">
         <v>946</v>
       </c>
-      <c r="B139" t="s">
+      <c r="C139" t="s">
         <v>947</v>
       </c>
-      <c r="C139" t="s">
+      <c r="D139" t="s">
         <v>948</v>
       </c>
-      <c r="D139" t="s">
+      <c r="E139" t="s">
         <v>949</v>
       </c>
-      <c r="E139" t="s">
+      <c r="F139" t="s">
         <v>950</v>
       </c>
-      <c r="F139" t="s">
+      <c r="G139" t="s">
         <v>951</v>
       </c>
-      <c r="G139" t="s">
-        <v>952</v>
-      </c>
       <c r="H139" t="s">
-        <v>1038</v>
+        <v>1037</v>
       </c>
       <c r="I139" t="s">
         <v>7</v>
@@ -8029,28 +8029,28 @@
     </row>
     <row r="140" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A140" t="s">
+        <v>952</v>
+      </c>
+      <c r="B140" t="s">
         <v>953</v>
       </c>
-      <c r="B140" t="s">
+      <c r="C140" t="s">
         <v>954</v>
       </c>
-      <c r="C140" t="s">
+      <c r="D140" t="s">
         <v>955</v>
       </c>
-      <c r="D140" t="s">
+      <c r="E140" t="s">
         <v>956</v>
       </c>
-      <c r="E140" t="s">
+      <c r="F140" t="s">
         <v>957</v>
       </c>
-      <c r="F140" t="s">
+      <c r="G140" t="s">
         <v>958</v>
       </c>
-      <c r="G140" t="s">
-        <v>959</v>
-      </c>
       <c r="H140" t="s">
-        <v>1045</v>
+        <v>1044</v>
       </c>
       <c r="I140" t="s">
         <v>16</v>
@@ -8061,28 +8061,28 @@
     </row>
     <row r="141" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="A141" t="s">
+        <v>959</v>
+      </c>
+      <c r="B141" t="s">
         <v>960</v>
       </c>
-      <c r="B141" t="s">
+      <c r="C141" t="s">
         <v>961</v>
       </c>
-      <c r="C141" t="s">
+      <c r="D141" t="s">
         <v>962</v>
       </c>
-      <c r="D141" t="s">
+      <c r="E141" t="s">
         <v>963</v>
       </c>
-      <c r="E141" t="s">
+      <c r="F141" t="s">
         <v>964</v>
       </c>
-      <c r="F141" t="s">
+      <c r="G141" t="s">
         <v>965</v>
       </c>
-      <c r="G141" t="s">
-        <v>966</v>
-      </c>
       <c r="H141" t="s">
-        <v>1041</v>
+        <v>1040</v>
       </c>
       <c r="I141" t="s">
         <v>7</v>

</xml_diff>